<commit_message>
Add worked coding example (P2) and fix a participant-label collision
Fixes a real bug in the codebook template: the example row and the
blank fill-in rows both started at "P1", colliding. Renamed the example
row to "P-ej (ejemplo)" across Cobertura protocolo, Ancla objetivación,
and Reflexividad.

Adds a full worked example coding the researcher's second interview
(anonymized as P2, real name not preserved) against codebook v0:
per-código evidence with timestamps, one inductive code proposed
(preocupacion_recursos_materiales_infraestructura), and an honest gap
flag on the Bloque 3 objetivación anchor (not clearly administered in
this transcript). Reflected into the Excel workbook as a distinct demo
file (codebook_v0_EJEMPLO_P2.xlsx) alongside the blank master template.
Does NOT commit the raw interview transcript -- pending a decision on
whether that's appropriate given the informed-consent protocol.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -1006,6 +1006,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -2206,6 +2208,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -2256,7 +2260,7 @@
     <row r="6">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>P1 (ejemplo)</t>
+          <t>P-ej (ejemplo)</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
@@ -2606,6 +2610,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -2626,7 +2632,7 @@
     <row r="6">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>P1 (ejemplo)</t>
+          <t>P-ej (ejemplo)</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Consolidate to a single working codebook; add Segmentos codificados
Adds a 12th sheet, "Segmentos codificados" -- one row per coded
fragment across all interviews (Participante, Bloque, Código(s), Cita
textual, Notas), filterable by participant or code. Seeded with the 9
real coded segments from P2 (Entrevista 2).

Retires codebook_v0_EJEMPLO_P2.xlsx as a separate file: the researcher
should work from one single file going forward, not one codebook per
interview. This master now IS that file, with P2 already loaded as the
first real coded case across all relevant sheets (Cobertura protocolo,
Ancla objetivación, Log códigos inductivos, Saturación, Segmentos
codificados).
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -14,10 +14,11 @@
     <sheet name="Núcleo 4" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Marcadores imaginario" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Log códigos inductivos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Cobertura protocolo" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Ancla objetivación" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Saturación" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Reflexividad" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Segmentos codificados" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Cobertura protocolo" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Ancla objetivación" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Saturación" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Reflexividad" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -80,7 +81,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +124,12 @@
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+        <bgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -150,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -213,6 +220,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -715,6 +728,220 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ancla privilegiada — Bloque 3, Pregunta 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuando la entrevista incluya "¿Qué sabés sobre la IAG? Si tuvieras que explicarle a alguien qué es, cómo se lo explicarías?", tratá la primera metáfora/imagen espontánea como dato de mayor peso para objetivacion_imagen_concreta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Participante</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>¿Se administró Bloque 3, P1? (Sí/No)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Primera metáfora/imagen espontánea</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>P-ej (ejemplo)</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>"Es como tener un asistente que te ayuda a armar cosas rápido"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n"/>
+      <c r="C7" s="18" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>No queda claro (ver nota)</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>No se identifica una metáfora espontánea clara. La entrevistadora preguntó qué recurso/app usó (identificación de herramienta), no una definición espontánea del concepto IAG.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="n"/>
+      <c r="C12" s="18" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="18" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n"/>
+      <c r="C14" s="18" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="18" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n"/>
+      <c r="C16" s="18" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n"/>
+      <c r="C18" s="18" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="18" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="n"/>
+      <c r="C20" s="18" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="n"/>
+      <c r="C21" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -788,14 +1015,26 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="23">
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>1 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta (ausente-hallazgo), anclaje_tecnologia_previa, potencia_integracion_sustantiva, competencia_tecnica_declarada, competencia_critica_reflexiva, relacion_no_lineal_competencia_representacion, eco_discurso_institucional, voz_experiencial_propia, preocupacion_recursos_materiales_infraestructura (inductivo)</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="E7" s="25">
         <f>SUM($D$6:D7)</f>
         <v/>
       </c>
@@ -977,7 +1216,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1006,8 +1245,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -1990,12 +2227,32 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="18" t="n"/>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>preocupacion_recursos_materiales_infraestructura</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Preocupación explícita por falta de recursos materiales/infraestructura (equipamiento, conectividad, tiempo de la facilitadora) como barrera -- distinta de falta de formación en sí.</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>Núcleo 4 (matiz nuevo, distinto de 'brecha de formación')</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="n"/>
@@ -2175,6 +2432,754 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Segmentos codificados (registro de trabajo, todas las entrevistas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Una fila por cada fragmento que codifiques, de cualquier entrevista. Se puede filtrar por Participante o por Código para revisar todos los ejemplos de una categoría.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Participante</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Bloque</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Código(s)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Cita textual (breve)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>P-ej</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>competencia_tecnica_declarada</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>"Uso el celular para todo pero la compu me cuesta más"</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Fila de ejemplo — borrar antes de usar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>anclaje_tecnologia_previa</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>"con Canva, con otras aplicaciones que hay para hacer videos" [00:47]</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>Ancla la IAG en su relación previa con tecnología educativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>anclaje_tecnologia_previa</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>"Hay una en Google que dice gratuita" [06:11] (sobre Gemini)</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>Ancla la herramienta nueva en el ecosistema Google ya conocido</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>competencia_tecnica_declarada</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>"A mí me encanta explorar, me encanta aprender" [02:50]</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>competencia_tecnica_declarada + relacion_no_lineal_competencia_representacion</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>"todavía no la he ni la he explorado, sinceramente. Sería mentirte si te digo que hice algo" [01:16]</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>Alta competencia tecnológica general declarada, pero baja exposición práctica específica a IAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>"le ponemos los nombres"... "vamos aplicando lo que nosotros trabajamos" [04:47]</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>Agrega su propia capa pedagógica a la propuesta de la facilitadora, no la sigue sin más</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>voz_experiencial_propia</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>Relato completo de la actividad con la facilitadora (dibujos del cuerpo humano) [01:43]-[02:33]</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>Episodio concreto y situado, no eco institucional</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>"el docente tiene que aprender, tiene que actualizarse" [10:40]</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>Marcador: necesidad de formación/capacitación</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>potencia_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>"con la IA para poder hacer las evaluaciones más rápidas" [12:12]</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>preocupacion_recursos_materiales_infraestructura (inductivo)</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>"tablets viejas"... "tengo que pedir prestada" [18:40]-[19:39]</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>Código inductivo nuevo — ver Log códigos inductivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="18" t="n"/>
+      <c r="D15" s="18" t="n"/>
+      <c r="E15" s="18" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="18" t="n"/>
+      <c r="B16" s="18" t="n"/>
+      <c r="C16" s="18" t="n"/>
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="18" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="18" t="n"/>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="18" t="n"/>
+      <c r="B18" s="18" t="n"/>
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="n"/>
+      <c r="E18" s="18" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="18" t="n"/>
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="18" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="18" t="n"/>
+      <c r="B20" s="18" t="n"/>
+      <c r="C20" s="18" t="n"/>
+      <c r="D20" s="18" t="n"/>
+      <c r="E20" s="18" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="18" t="n"/>
+      <c r="B21" s="18" t="n"/>
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+      <c r="E21" s="18" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="18" t="n"/>
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="18" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="18" t="n"/>
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="18" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="18" t="n"/>
+      <c r="B24" s="18" t="n"/>
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="18" t="n"/>
+      <c r="E24" s="18" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="18" t="n"/>
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="18" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="18" t="n"/>
+      <c r="B26" s="18" t="n"/>
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="18" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="18" t="n"/>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="18" t="n"/>
+      <c r="B28" s="18" t="n"/>
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="18" t="n"/>
+      <c r="E28" s="18" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="18" t="n"/>
+      <c r="B29" s="18" t="n"/>
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="18" t="n"/>
+      <c r="E29" s="18" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="18" t="n"/>
+      <c r="B30" s="18" t="n"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="18" t="n"/>
+      <c r="B31" s="18" t="n"/>
+      <c r="C31" s="18" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="18" t="n"/>
+      <c r="B32" s="18" t="n"/>
+      <c r="C32" s="18" t="n"/>
+      <c r="D32" s="18" t="n"/>
+      <c r="E32" s="18" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="18" t="n"/>
+      <c r="B33" s="18" t="n"/>
+      <c r="C33" s="18" t="n"/>
+      <c r="D33" s="18" t="n"/>
+      <c r="E33" s="18" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="18" t="n"/>
+      <c r="B34" s="18" t="n"/>
+      <c r="C34" s="18" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="18" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="18" t="n"/>
+      <c r="B35" s="18" t="n"/>
+      <c r="C35" s="18" t="n"/>
+      <c r="D35" s="18" t="n"/>
+      <c r="E35" s="18" t="n"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="18" t="n"/>
+      <c r="B36" s="18" t="n"/>
+      <c r="C36" s="18" t="n"/>
+      <c r="D36" s="18" t="n"/>
+      <c r="E36" s="18" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="18" t="n"/>
+      <c r="B37" s="18" t="n"/>
+      <c r="C37" s="18" t="n"/>
+      <c r="D37" s="18" t="n"/>
+      <c r="E37" s="18" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="18" t="n"/>
+      <c r="B38" s="18" t="n"/>
+      <c r="C38" s="18" t="n"/>
+      <c r="D38" s="18" t="n"/>
+      <c r="E38" s="18" t="n"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="18" t="n"/>
+      <c r="B39" s="18" t="n"/>
+      <c r="C39" s="18" t="n"/>
+      <c r="D39" s="18" t="n"/>
+      <c r="E39" s="18" t="n"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="18" t="n"/>
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="18" t="n"/>
+      <c r="D40" s="18" t="n"/>
+      <c r="E40" s="18" t="n"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="18" t="n"/>
+      <c r="B41" s="18" t="n"/>
+      <c r="C41" s="18" t="n"/>
+      <c r="D41" s="18" t="n"/>
+      <c r="E41" s="18" t="n"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="18" t="n"/>
+      <c r="B42" s="18" t="n"/>
+      <c r="C42" s="18" t="n"/>
+      <c r="D42" s="18" t="n"/>
+      <c r="E42" s="18" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="18" t="n"/>
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="18" t="n"/>
+      <c r="D43" s="18" t="n"/>
+      <c r="E43" s="18" t="n"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="18" t="n"/>
+      <c r="B44" s="18" t="n"/>
+      <c r="C44" s="18" t="n"/>
+      <c r="D44" s="18" t="n"/>
+      <c r="E44" s="18" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="18" t="n"/>
+      <c r="B45" s="18" t="n"/>
+      <c r="C45" s="18" t="n"/>
+      <c r="D45" s="18" t="n"/>
+      <c r="E45" s="18" t="n"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="18" t="n"/>
+      <c r="B46" s="18" t="n"/>
+      <c r="C46" s="18" t="n"/>
+      <c r="D46" s="18" t="n"/>
+      <c r="E46" s="18" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="18" t="n"/>
+      <c r="B47" s="18" t="n"/>
+      <c r="C47" s="18" t="n"/>
+      <c r="D47" s="18" t="n"/>
+      <c r="E47" s="18" t="n"/>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="18" t="n"/>
+      <c r="B48" s="18" t="n"/>
+      <c r="C48" s="18" t="n"/>
+      <c r="D48" s="18" t="n"/>
+      <c r="E48" s="18" t="n"/>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="18" t="n"/>
+      <c r="B49" s="18" t="n"/>
+      <c r="C49" s="18" t="n"/>
+      <c r="D49" s="18" t="n"/>
+      <c r="E49" s="18" t="n"/>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="18" t="n"/>
+      <c r="B50" s="18" t="n"/>
+      <c r="C50" s="18" t="n"/>
+      <c r="D50" s="18" t="n"/>
+      <c r="E50" s="18" t="n"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="18" t="n"/>
+      <c r="B51" s="18" t="n"/>
+      <c r="C51" s="18" t="n"/>
+      <c r="D51" s="18" t="n"/>
+      <c r="E51" s="18" t="n"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="18" t="n"/>
+      <c r="B52" s="18" t="n"/>
+      <c r="C52" s="18" t="n"/>
+      <c r="D52" s="18" t="n"/>
+      <c r="E52" s="18" t="n"/>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="18" t="n"/>
+      <c r="B53" s="18" t="n"/>
+      <c r="C53" s="18" t="n"/>
+      <c r="D53" s="18" t="n"/>
+      <c r="E53" s="18" t="n"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="18" t="n"/>
+      <c r="B54" s="18" t="n"/>
+      <c r="C54" s="18" t="n"/>
+      <c r="D54" s="18" t="n"/>
+      <c r="E54" s="18" t="n"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="18" t="n"/>
+      <c r="B55" s="18" t="n"/>
+      <c r="C55" s="18" t="n"/>
+      <c r="D55" s="18" t="n"/>
+      <c r="E55" s="18" t="n"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="18" t="n"/>
+      <c r="B56" s="18" t="n"/>
+      <c r="C56" s="18" t="n"/>
+      <c r="D56" s="18" t="n"/>
+      <c r="E56" s="18" t="n"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="18" t="n"/>
+      <c r="B57" s="18" t="n"/>
+      <c r="C57" s="18" t="n"/>
+      <c r="D57" s="18" t="n"/>
+      <c r="E57" s="18" t="n"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="18" t="n"/>
+      <c r="B58" s="18" t="n"/>
+      <c r="C58" s="18" t="n"/>
+      <c r="D58" s="18" t="n"/>
+      <c r="E58" s="18" t="n"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="18" t="n"/>
+      <c r="B59" s="18" t="n"/>
+      <c r="C59" s="18" t="n"/>
+      <c r="D59" s="18" t="n"/>
+      <c r="E59" s="18" t="n"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="18" t="n"/>
+      <c r="B60" s="18" t="n"/>
+      <c r="C60" s="18" t="n"/>
+      <c r="D60" s="18" t="n"/>
+      <c r="E60" s="18" t="n"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="18" t="n"/>
+      <c r="B61" s="18" t="n"/>
+      <c r="C61" s="18" t="n"/>
+      <c r="D61" s="18" t="n"/>
+      <c r="E61" s="18" t="n"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="18" t="n"/>
+      <c r="B62" s="18" t="n"/>
+      <c r="C62" s="18" t="n"/>
+      <c r="D62" s="18" t="n"/>
+      <c r="E62" s="18" t="n"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="18" t="n"/>
+      <c r="B63" s="18" t="n"/>
+      <c r="C63" s="18" t="n"/>
+      <c r="D63" s="18" t="n"/>
+      <c r="E63" s="18" t="n"/>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="18" t="n"/>
+      <c r="B64" s="18" t="n"/>
+      <c r="C64" s="18" t="n"/>
+      <c r="D64" s="18" t="n"/>
+      <c r="E64" s="18" t="n"/>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="18" t="n"/>
+      <c r="B65" s="18" t="n"/>
+      <c r="C65" s="18" t="n"/>
+      <c r="D65" s="18" t="n"/>
+      <c r="E65" s="18" t="n"/>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="18" t="n"/>
+      <c r="B66" s="18" t="n"/>
+      <c r="C66" s="18" t="n"/>
+      <c r="D66" s="18" t="n"/>
+      <c r="E66" s="18" t="n"/>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="18" t="n"/>
+      <c r="B67" s="18" t="n"/>
+      <c r="C67" s="18" t="n"/>
+      <c r="D67" s="18" t="n"/>
+      <c r="E67" s="18" t="n"/>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="18" t="n"/>
+      <c r="B68" s="18" t="n"/>
+      <c r="C68" s="18" t="n"/>
+      <c r="D68" s="18" t="n"/>
+      <c r="E68" s="18" t="n"/>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="18" t="n"/>
+      <c r="B69" s="18" t="n"/>
+      <c r="C69" s="18" t="n"/>
+      <c r="D69" s="18" t="n"/>
+      <c r="E69" s="18" t="n"/>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="18" t="n"/>
+      <c r="B70" s="18" t="n"/>
+      <c r="C70" s="18" t="n"/>
+      <c r="D70" s="18" t="n"/>
+      <c r="E70" s="18" t="n"/>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="18" t="n"/>
+      <c r="B71" s="18" t="n"/>
+      <c r="C71" s="18" t="n"/>
+      <c r="D71" s="18" t="n"/>
+      <c r="E71" s="18" t="n"/>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="18" t="n"/>
+      <c r="B72" s="18" t="n"/>
+      <c r="C72" s="18" t="n"/>
+      <c r="D72" s="18" t="n"/>
+      <c r="E72" s="18" t="n"/>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="18" t="n"/>
+      <c r="B73" s="18" t="n"/>
+      <c r="C73" s="18" t="n"/>
+      <c r="D73" s="18" t="n"/>
+      <c r="E73" s="18" t="n"/>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="18" t="n"/>
+      <c r="B74" s="18" t="n"/>
+      <c r="C74" s="18" t="n"/>
+      <c r="D74" s="18" t="n"/>
+      <c r="E74" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2208,8 +3213,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -2321,20 +3324,48 @@
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B8" s="22" t="n"/>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
-      <c r="F8" s="22" t="n"/>
-      <c r="G8" s="22" t="n"/>
-      <c r="H8" s="22" t="n"/>
-      <c r="I8" s="23">
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E8" s="25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F8" s="25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H8" s="25" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I8" s="25">
         <f>COUNTIF(B8:H8,"Sí")</f>
         <v/>
       </c>
@@ -2580,212 +3611,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ancla privilegiada — Bloque 3, Pregunta 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuando la entrevista incluya "¿Qué sabés sobre la IAG? Si tuvieras que explicarle a alguien qué es, cómo se lo explicarías?", tratá la primera metáfora/imagen espontánea como dato de mayor peso para objetivacion_imagen_concreta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Participante</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>¿Se administró Bloque 3, P1? (Sí/No)</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Primera metáfora/imagen espontánea</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>P-ej (ejemplo)</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>"Es como tener un asistente que te ayuda a armar cosas rápido"</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="18" t="n"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>P14</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="21" t="inlineStr">
-        <is>
-          <t>P15</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="18" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Replace provisional imaginary markers (v0) with real primary sources (v1)
The researcher shared full text of the 4 official documents that
constitute the "imaginario oficial" corpus at three levels: UNESCO
(Holmes et al. 2021, global), Nación (Ministerio de Capital Humano
2025), and CABA (Ministerio de Educación GCBA -- "Guía para un uso
crítico" + its companion "Marco de gobernanza"). This closes the 403
proxy-block gap from the earlier literature search.

Rebuilds the marker list (codebook_v0_manual.md and the Excel
"Marcadores imaginario" sheet) with 14 markers pulled directly from the
primary texts, organized by level, each traceable to a specific
document/section. Updates domain-profile.md's data source entry to
reflect these are now in-hand, fully read documents rather than a
pending item.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -157,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -228,6 +228,7 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1907,213 +1908,358 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Lista de marcadores v0 del imaginario oficial (provisoria)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>Lista de marcadores v1 del imaginario oficial (fuentes primarias, 3 niveles)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Extraída de una primera lectura de la Guía 2025 (PaideIA) y el informe Educ.ar 2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>IMPORTANTE: el acceso directo a la Guía 2025 estuvo bloqueado durante la búsqueda bibliográfica (error 403 del proxy hacia el dominio .gob.ar). Esta lista se armó con lo confirmado por fuentes secundarias y debe revisarse/completarse cuando puedas leer el documento completo vos misma. Es un instrumento vivo: agregá marcadores nuevos a medida que codificás, con fecha, en las filas amarillas de abajo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+          <t>Reemplaza la v0 (fuentes secundarias). Fuentes primarias completas en master_supporting_docs/supporting_papers/: UNESCO_Holmes_2021_IA_educacion.pdf (global), Guia_Nacion_Integracion_IA_Educacion_2025.pdf (nación), Guia_CABA_uso_critico_v2.pdf + Marco_gobernanza_CABA_IA.pdf (jurisdiccional -- tu propio sitio de investigación).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
         <is>
           <t>Marcador</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Documento fuente</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Notas / dónde apareció</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>aprendizaje personalizado</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Guía 2025 / Educ.ar (confirmar página exacta)</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>v0 — provisorio</t>
-        </is>
-      </c>
-      <c r="D7" s="17" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>acompañamiento docente (no reemplazo)</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Guía 2025 / Educ.ar (confirmar página exacta)</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>v0 — provisorio</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>uso responsable/ético</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Guía 2025 / Educ.ar (confirmar página exacta)</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>v0 — provisorio</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>necesidad de formación/capacitación</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Guía 2025 / Educ.ar (confirmar página exacta)</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>v0 — provisorio</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>brecha de formación</t>
-        </is>
-      </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>Guía 2025 / Educ.ar (confirmar página exacta)</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="inlineStr">
-        <is>
-          <t>v0 — provisorio</t>
-        </is>
-      </c>
-      <c r="D11" s="17" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>integración progresiva</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>Guía 2025 / Educ.ar (confirmar página exacta)</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>v0 — provisorio</t>
-        </is>
-      </c>
-      <c r="D12" s="17" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>eficiencia</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>Guía 2025 / Educ.ar (confirmar página exacta)</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>v0 — provisorio</t>
-        </is>
-      </c>
-      <c r="D13" s="17" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="n"/>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="18" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="n"/>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="n"/>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="18" t="n"/>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="18" t="n"/>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Nivel</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>Cita/paráfrasis y nota de uso</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>"uso responsable, ético y efectivo" / "uso crítico, ético y creativo"</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Nación/CABA</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Guía Nación p.5; Guía CABA p.4</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Formulación casi idéntica en ambos niveles -- alta frecuencia esperada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>"acompañar" / "acompañamiento docente" (no reemplazo)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Nación/CABA</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Guía Nación §Impacto en el rol docente; Marco gobernanza CABA, principio 1</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>"la IA nunca reemplaza... complementa la labor docente sin sustituir el contacto humano"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>"potenciar lo humano, no reemplazarlo con IA"</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>CABA</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Guía CABA p.6, principio 'Humanismo digital'</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Principio orientador explícito</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>"el docente tiene que aprender, tiene que actualizarse" / "formación continua"</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Nación/CABA</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Guía Nación §Estrategias de capacitación; Marco gobernanza CABA, Nivel docentes</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Ya identificado en la entrevista de P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>"reducir la carga administrativa" (para tareas de mayor valor pedagógico)</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>CABA</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Marco gobernanza CABA, Nivel docentes, objetivos específicos</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Muy específico -- buen candidato cuando la docente habla de ahorrar tiempo en corrección/evaluación</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>"eficiencia" / "agilizar la corrección" / "ahorro de tiempo"</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Nación/CABA</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Guía Nación §Evaluación y retroalimentación; Guía CABA p.5</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Ya usado en P2 ("evaluaciones más rápidas")</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>"personalización" / "educación personalizada" / "adaptar al ritmo de cada estudiante"</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Presente casi textual en los 3 documentos</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Marcador transversal -- altísima frecuencia esperada</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>"sesgos" / "sesgo algorítmico" / "alucinaciones"</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Nación/CABA</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>Guía Nación p.8; Guía CABA glosario</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Vocabulario técnico -- si la docente lo usa tal cual, eco fuerte, no genuino desde la experiencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>"brecha(s)" -- acceso, formación, infraestructura, digital</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Guía Nación p.8; Marco gobernanza CABA, Equidad e inclusión digital</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Distinguir del código inductivo de P2 (preocupacion_recursos_materiales_infraestructura) -- puede solaparse</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>"pensamiento crítico" / "las 4C" (creatividad, pensamiento crítico, comunicación, colaboración)</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>CABA</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Guía CABA p.5</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Vocabulario específico de la Guía CABA -- alta especificidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>"protección de datos" / "consentimiento informado" / "privacidad"</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Presente en los 3, cita Ley 25.326 en Nación y CABA</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>Poco probable en discurso espontáneo sobre representaciones, pero vigilar</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>"aliada estratégica" / "IA como aliada"</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>CABA</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Marco gobernanza CABA, Presentación</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Metáfora oficial específica -- marcador fuerte si aparece "aliada"</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>"estrategias auténticas que promuevan aprendizajes que no puedan ser automatizados" / "palabra propia"</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>CABA/Nación</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Marco gobernanza CABA, Nivel docentes; Guía Nación p.18-19 (Ravela y Cardoner)</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>Vocabulario de evaluación auténtica -- vigilar en el eje de aprendizaje significativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>"criterio docente" / "supervisión docente" / "el docente valida y decide"</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Marco gobernanza CABA, principio 5; Guía Nación (rol del docente como mediador)</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Formulación de resguardo del rol, distinta de "no reemplaza" -- vigilar matices</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="n"/>
@@ -2133,10 +2279,81 @@
       <c r="C21" s="18" t="n"/>
       <c r="D21" s="18" t="n"/>
     </row>
+    <row r="22">
+      <c r="A22" s="18" t="n"/>
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="n"/>
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="n"/>
+      <c r="B24" s="18" t="n"/>
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="18" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n"/>
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="n"/>
+      <c r="B26" s="18" t="n"/>
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="n"/>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="n"/>
+      <c r="B28" s="18" t="n"/>
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="18" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="n"/>
+      <c r="B29" s="18" t="n"/>
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="18" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="n"/>
+      <c r="B30" s="18" t="n"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="n"/>
+      <c r="B31" s="18" t="n"/>
+      <c r="C31" s="18" t="n"/>
+      <c r="D31" s="18" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="n"/>
+      <c r="B32" s="18" t="n"/>
+      <c r="C32" s="18" t="n"/>
+      <c r="D32" s="18" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="n"/>
+      <c r="B33" s="18" t="n"/>
+      <c r="C33" s="18" t="n"/>
+      <c r="D33" s="18" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A4:D4"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Verify Castañeda et al. (2025) citation, resolve all UNVERIFIED flags
Researcher shared the full text: Castañeda, Postigo-Fuentes &
Arroyo-Sagasta (2025), "Beyond Tools, Toward Power Structures: A
Critical Review of AI in Primary Education," REEC 48 (extra), 73-95.
Same special issue as Fuertes-Alpiste and Estormovski (already in the
bibliography) but with a primary-education-specific focus and a
7-dimension critical framework (instrumental/epistemological/ethical/
social/political/commercial/ideological) -- a new literature find, not
previously surfaced.

Adds the verified BibTeX entry, replaces every "% UNVERIFIED" flag
across the manual codebook, the Excel workbook (Núcleo 4 and Núcleo 5
sheets), and domain-profile.md, and adds it to antecedentes.md as a
relevant primary-education-specific antecedent.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -2265,6 +2265,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2272,6 +2273,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -2370,7 +2372,7 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Habla de brecha pública/privada, con/sin recursos, como condición que la IA no resuelve o profundiza. Ej.: "Las que ya tienen todo van a poder usarla, las que no van a quedar más atrás". Distinguir de preocupacion_recursos_materiales_infraestructura (inductivo P2): esa es concreta/propia, esta es estructural/comparativa -- pueden coexistir. Ref.: Saura et al. (2024); Castañeda et al. (2025) [UNVERIFIED -- no está en la bibliografía].</t>
+          <t>Habla de brecha pública/privada, con/sin recursos, como condición que la IA no resuelve o profundiza. Ej.: "Las que ya tienen todo van a poder usarla, las que no van a quedar más atrás". Distinguir de preocupacion_recursos_materiales_infraestructura (inductivo P2): esa es concreta/propia, esta es estructural/comparativa -- pueden coexistir. Ref.: Saura et al. (2024); Castañeda, Postigo-Fuentes &amp; Arroyo-Sagasta (2025, REEC 48 extra) -- verificada.</t>
         </is>
       </c>
     </row>
@@ -2429,6 +2431,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
@@ -2513,7 +2516,7 @@
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>"La uso para hacer los comentarios del boletín". Puede coexistir con eco_discurso_institucional (marcador "reducir la carga administrativa", Marco gobernanza CABA). Registrar si distingue estos usos de los usos pedagógicos con alumnos. Ref.: Castañeda et al. (2025) [UNVERIFIED]; Cabello (2006).</t>
+          <t>"La uso para hacer los comentarios del boletín". Puede coexistir con eco_discurso_institucional (marcador "reducir la carga administrativa", Marco gobernanza CABA). Registrar si distingue estos usos de los usos pedagógicos con alumnos. Ref.: Castañeda, Postigo-Fuentes &amp; Arroyo-Sagasta (2025, REEC 48 extra) -- verificada; Cabello (2006).</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2538,7 @@
       </c>
       <c r="D8" s="28" t="inlineStr">
         <is>
-          <t>"Me gusta que mis planificaciones sean mías". Código de alta carga identitaria -- anotar si la tensión se resuelve a favor de la IA, de la docente, o queda sin resolver. Puede coexistir con competencia_critica_reflexiva (Núcleo 3). Ref.: Moscovici (1986); Castañeda et al. (2025) [UNVERIFIED].</t>
+          <t>"Me gusta que mis planificaciones sean mías". Código de alta carga identitaria -- anotar si la tensión se resuelve a favor de la IA, de la docente, o queda sin resolver. Puede coexistir con competencia_critica_reflexiva (Núcleo 3). Ref.: Moscovici (1986); Castañeda, Postigo-Fuentes &amp; Arroyo-Sagasta (2025, REEC 48 extra) -- verificada.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Núcleo 5 to strategy memo (Revision 4) and test codebook v0 against P2/P3/P4
Strategist formally integrated the researcher-proposed 5th núcleo (diseño
didáctico y uso pedagógico) and 3 new imaginarios codes into the approved
strategy memo, pseudo_code.md, and decision record.

Codebook v0 tested against 3 real interviews (P2, P3, P4): no codes
required forcing, previously-absent codes (objetivacion_imagen_concreta,
anclaje_figura_humana) appeared cleanly in later cases confirming real
variation rather than broken specification, and the new Núcleo 5 rendered
immediately with a near-textbook match. Two inductive code candidates
logged for researcher validation. Excel workbook updated with P3/P4
tracking data. Raw interview transcripts remain local-only (gitignored),
per the project's data-privacy convention.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -164,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -241,6 +241,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -928,37 +931,93 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B9" s="22" t="n"/>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="22" t="n"/>
-      <c r="E9" s="22" t="n"/>
-      <c r="F9" s="22" t="n"/>
-      <c r="G9" s="22" t="n"/>
-      <c r="H9" s="22" t="n"/>
-      <c r="I9" s="23">
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H9" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I9" s="29">
         <f>COUNTIF(B9:H9,"Sí")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="B10" s="22" t="n"/>
-      <c r="C10" s="22" t="n"/>
-      <c r="D10" s="22" t="n"/>
-      <c r="E10" s="22" t="n"/>
-      <c r="F10" s="22" t="n"/>
-      <c r="G10" s="22" t="n"/>
-      <c r="H10" s="22" t="n"/>
-      <c r="I10" s="23">
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F10" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H10" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I10" s="29">
         <f>COUNTIF(B10:H10,"Sí")</f>
         <v/>
       </c>
@@ -1259,22 +1318,38 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>"Es un recurso accesible para poder... esas ideas que alguien tiene... lo que hace la inteligencia... es ayudarte a organizar esa idea y darte otras cosas que capaz no las tenías en cuenta" [06:54]-[07:24]</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>"Es... un lenguaje... en el cual el ser humano puede incorporar determinada información... y esa inteligencia responde en relación a eso con la cual fue cargada" [08:18]-[08:59]</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="21" t="inlineStr">
@@ -1488,25 +1563,49 @@
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="23">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>2 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta (primera instancia positiva), imaginario_inevitabilidad_tecnologica (caso negativo/matizado), imaginario_rol_docente_futuro, criterio_sentido_pedagogico, criterio_contextual_grupo, eco_de_par_colega (inductivo candidato)</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="25">
         <f>SUM($D$6:D8)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="23" t="n">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>3 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>anclaje_figura_humana (primera instancia limpia), uso_iai_apoyo_administrativo, mito_estigma_pereza (inductivo candidato) -- imaginario_inevitabilidad_tecnologica ya visto en P3 pero con polaridad nueva (afirmativa), no contado en el total</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="23">
+      <c r="E9" s="25">
         <f>SUM($D$6:D9)</f>
         <v/>
       </c>
@@ -2265,7 +2364,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2273,7 +2371,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
@@ -2431,7 +2528,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
@@ -3121,18 +3217,58 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="n"/>
-      <c r="B8" s="18" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="18" t="n"/>
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>eco_de_par_colega</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>Representación mediada por un tercero (colega/formador/a) relatada por la participante -- distinta de voz_experiencial_propia (no es experiencia directa) y de eco_discurso_institucional (no viene de un documento oficial).</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Núcleo 4 (candidato -- en observación, n=1)</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="n"/>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>mito_estigma_pereza</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Referencia al estigma social/moral de que usar IA es "de vagos" o de facilismo -- distinto de imaginario_inevitabilidad_tecnologica (no es sobre si va a pasar) y de imaginario_rol_docente_futuro (no es sobre el rol futuro, es un juicio social presente).</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Núcleo 4 (candidato -- en observación, n=1)</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="18" t="n"/>
@@ -3617,158 +3753,562 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="18" t="n"/>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n"/>
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
+        <is>
+          <t>"siempre miro lo que es el grupo de chicos" [03:40]-[04:36]</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="inlineStr">
+        <is>
+          <t>Decide uso de tecnología en función del grupo real, no del docente</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="18" t="n"/>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>"es un recurso accesible... te organiza esa idea" [06:54]-[07:24]</t>
+        </is>
+      </c>
+      <c r="E16" s="29" t="inlineStr">
+        <is>
+          <t>Primera objetivación positiva del corpus (ausente en P2)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="18" t="n"/>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico + criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="inlineStr">
+        <is>
+          <t>Armó secuencia de "seres vivos" con NotebookLM para ayudar a una colega, a partir del diseño curricular [08:20]-[09:30]</t>
+        </is>
+      </c>
+      <c r="E17" s="29" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="18" t="n"/>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>eco_de_par_colega (inductivo candidato)</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="inlineStr">
+        <is>
+          <t>Relato de la preocupación de una profesora universitaria sobre estudiantes que usan IA "sin conciencia" [09:40]-[10:52]</t>
+        </is>
+      </c>
+      <c r="E18" s="29" t="inlineStr">
+        <is>
+          <t>Representación mediada por un tercero — no es voz propia ni eco institucional; ver Log códigos inductivos</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="18" t="n"/>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="inlineStr">
+        <is>
+          <t>"nos puede ayudar pero siendo prolijos y teniendo una planificación con la IA, y en qué momento, no en cualquier momento" [13:07]-[13:36]</t>
+        </is>
+      </c>
+      <c r="E19" s="29" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="18" t="n"/>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
-      <c r="E20" s="18" t="n"/>
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_rol_docente_futuro</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>"tiene que ir acompañado... el docente un poquito más adelante que la inteligencia" [13:36]-[14:02]</t>
+        </is>
+      </c>
+      <c r="E20" s="29" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="18" t="n"/>
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="18" t="n"/>
-      <c r="E21" s="18" t="n"/>
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>uso_iai_apoyo_administrativo (evaluado, no aplica) / criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D21" s="29" t="inlineStr">
+        <is>
+          <t>Ayudó a armar secuencia + evaluación completa para colegas; pidió adaptar evaluación para alumna con dificultades, IA generó versión de desarrollo [14:59]-[15:46]</t>
+        </is>
+      </c>
+      <c r="E21" s="29" t="inlineStr">
+        <is>
+          <t>No se codifica como apoyo_administrativo: es diseño didáctico completo, no tarea de gestión</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="18" t="n"/>
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="18" t="n"/>
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C22" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>"puede llegar a empeorar si el docente no se capacita... si están mal usadas, puede empeorar la educación" [16:27]-[16:48]</t>
+        </is>
+      </c>
+      <c r="E22" s="29" t="inlineStr">
+        <is>
+          <t>Caso negativo/matizado — condiciona la inevitabilidad a la formación docente</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="18" t="n"/>
-      <c r="B23" s="18" t="n"/>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
+        <is>
+          <t>"una capacitación" [16:48]; "le falta formación" [18:49]-[19:17]</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>Marcador: formación continua</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="18" t="n"/>
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="18" t="n"/>
-      <c r="E24" s="18" t="n"/>
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C24" s="29" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
+        <is>
+          <t>"hay que usarla con cuidado, no hay que enamorarse de la IA... hay que saber cuándo y para qué" [19:17]-[19:40]</t>
+        </is>
+      </c>
+      <c r="E24" s="29" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="18" t="n"/>
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="18" t="n"/>
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>competencia_tecnica_declarada</t>
+        </is>
+      </c>
+      <c r="D25" s="29" t="inlineStr">
+        <is>
+          <t>"lo uso para todo... desde el celu y si no bueno la compu" [03:20]-[04:45]</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="18" t="n"/>
-      <c r="B26" s="18" t="n"/>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="18" t="n"/>
-      <c r="E26" s="18" t="n"/>
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="inlineStr">
+        <is>
+          <t>"que se ensamble de manera correcta, que tenga una funcionalidad que sume... preguntarme a mí misma para qué la estoy incluyendo... un criterio razonable" [04:53]-[06:19]</t>
+        </is>
+      </c>
+      <c r="E26" s="29" t="inlineStr">
+        <is>
+          <t>Coincidencia casi textual con la definición del código</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="18" t="n"/>
-      <c r="B27" s="18" t="n"/>
-      <c r="C27" s="18" t="n"/>
-      <c r="D27" s="18" t="n"/>
-      <c r="E27" s="18" t="n"/>
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C27" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta</t>
+        </is>
+      </c>
+      <c r="D27" s="29" t="inlineStr">
+        <is>
+          <t>"es... un lenguaje... [que] responde en relación a [la información] con la cual fue cargada" [08:18]-[08:59]</t>
+        </is>
+      </c>
+      <c r="E27" s="29" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="18" t="n"/>
-      <c r="B28" s="18" t="n"/>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="18" t="n"/>
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="inlineStr">
+        <is>
+          <t>anclaje_figura_humana</t>
+        </is>
+      </c>
+      <c r="D28" s="29" t="inlineStr">
+        <is>
+          <t>"hoy en día yo creo que es mi asistente personal" [09:39]-[10:06]</t>
+        </is>
+      </c>
+      <c r="E28" s="29" t="inlineStr">
+        <is>
+          <t>Primera instancia limpia del corpus</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="18" t="n"/>
-      <c r="B29" s="18" t="n"/>
-      <c r="C29" s="18" t="n"/>
-      <c r="D29" s="18" t="n"/>
-      <c r="E29" s="18" t="n"/>
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C29" s="29" t="inlineStr">
+        <is>
+          <t>uso_iai_apoyo_administrativo</t>
+        </is>
+      </c>
+      <c r="D29" s="29" t="inlineStr">
+        <is>
+          <t>"para cualquier planificación que tenga que hacer... la utilizo para todo" [10:06]-[10:32]</t>
+        </is>
+      </c>
+      <c r="E29" s="29" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="18" t="n"/>
-      <c r="B30" s="18" t="n"/>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="18" t="n"/>
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C30" s="29" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva</t>
+        </is>
+      </c>
+      <c r="D30" s="29" t="inlineStr">
+        <is>
+          <t>"muchas veces el error está en la consigna de lo que se le pide al estudiante... no tanto en lo que hace el estudiante" [11:36]-[12:19]</t>
+        </is>
+      </c>
+      <c r="E30" s="29" t="inlineStr">
+        <is>
+          <t>Incluye reencuadre histórico ("Rincón del Vago") — relativiza el pánico moral sobre mal uso estudiantil</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="18" t="n"/>
-      <c r="B31" s="18" t="n"/>
-      <c r="C31" s="18" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="18" t="n"/>
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D31" s="29" t="inlineStr">
+        <is>
+          <t>"armar consignas que contribuyan al pensamiento crítico... no es mala palabra usarla... hay que usarla con criterio" [12:19]-[12:41]</t>
+        </is>
+      </c>
+      <c r="E31" s="29" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="18" t="n"/>
-      <c r="B32" s="18" t="n"/>
-      <c r="C32" s="18" t="n"/>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="18" t="n"/>
+      <c r="A32" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="inlineStr">
+        <is>
+          <t>criterio_contextual_grupo + criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D32" s="29" t="inlineStr">
+        <is>
+          <t>"se puede sumar tranquilamente a cualquier tipo de planificación... independientemente del grado" [12:41]-[13:44]</t>
+        </is>
+      </c>
+      <c r="E32" s="29" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="18" t="n"/>
-      <c r="B33" s="18" t="n"/>
-      <c r="C33" s="18" t="n"/>
-      <c r="D33" s="18" t="n"/>
-      <c r="E33" s="18" t="n"/>
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C33" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica</t>
+        </is>
+      </c>
+      <c r="D33" s="29" t="inlineStr">
+        <is>
+          <t>"va a ser parte de nuestras vidas más que nunca, más que ahora... ya es parte de nuestras vidas" [15:45]-[16:14]</t>
+        </is>
+      </c>
+      <c r="E33" s="29" t="inlineStr">
+        <is>
+          <t>Caso positivo, sin reservas — contrasta con el caso matizado de P3</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="18" t="n"/>
-      <c r="B34" s="18" t="n"/>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="18" t="n"/>
-      <c r="E34" s="18" t="n"/>
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B34" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D34" s="29" t="inlineStr">
+        <is>
+          <t>"empezar a capacitarse un poco más, a empezar a entender, a empezar a conocer" [16:14]-[16:36]</t>
+        </is>
+      </c>
+      <c r="E34" s="29" t="inlineStr">
+        <is>
+          <t>Marcador: formación continua</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="18" t="n"/>
-      <c r="B35" s="18" t="n"/>
-      <c r="C35" s="18" t="n"/>
-      <c r="D35" s="18" t="n"/>
-      <c r="E35" s="18" t="n"/>
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B35" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C35" s="29" t="inlineStr">
+        <is>
+          <t>mito_estigma_pereza (inductivo candidato)</t>
+        </is>
+      </c>
+      <c r="D35" s="29" t="inlineStr">
+        <is>
+          <t>"empezar a sacar algunos mitos, como por ejemplo que es de vagos usar la inteligencia" [16:36]-[17:04]</t>
+        </is>
+      </c>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>Estigma social del uso de IA — código inductivo candidato, n=1, ver Log códigos inductivos</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="18" t="n"/>
-      <c r="B36" s="18" t="n"/>
-      <c r="C36" s="18" t="n"/>
-      <c r="D36" s="18" t="n"/>
-      <c r="E36" s="18" t="n"/>
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_rol_docente_futuro</t>
+        </is>
+      </c>
+      <c r="D36" s="29" t="inlineStr">
+        <is>
+          <t>"el hecho de aportarle a los educadores el conocimiento también los estás empoderando... les estás abriendo nuevas puertas" [17:55]-[18:21]</t>
+        </is>
+      </c>
+      <c r="E36" s="29" t="inlineStr">
+        <is>
+          <t>No se propone código separado de "empoderamiento" — encaja en rol_docente_futuro</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="18" t="n"/>

</xml_diff>

<commit_message>
Code full interview corpus (P5-P13) against codebook v0 -- 13/13 done
Completes primary coding of all 13 transcribed interviews. Three codes
that looked underdeveloped with only 3 cases produced real instances once
the full corpus was coded (limita_integracion_sustantiva, imaginario_
desigualdad_estructural, tension_autoria_impronta). Two codes remain
genuinely weak across all 13, now a reportable finding rather than a gap.
Proposes a new inductive code (estrategia_deteccion_uso_estudiantil,
n=4) and strengthens an earlier candidate (eco_de_par_colega, n=2).
Last 4 interviews added no new axial categories -- early saturation
signal flagged for researcher confirmation. Raw transcripts anonymized
and kept local-only per the project's data-privacy convention.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -1023,163 +1023,415 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n"/>
-      <c r="C11" s="22" t="n"/>
-      <c r="D11" s="22" t="n"/>
-      <c r="E11" s="22" t="n"/>
-      <c r="F11" s="22" t="n"/>
-      <c r="G11" s="22" t="n"/>
-      <c r="H11" s="22" t="n"/>
-      <c r="I11" s="23">
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G11" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H11" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I11" s="29">
         <f>COUNTIF(B11:H11,"Sí")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="B12" s="22" t="n"/>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="22" t="n"/>
-      <c r="G12" s="22" t="n"/>
-      <c r="H12" s="22" t="n"/>
-      <c r="I12" s="23">
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E12" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G12" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H12" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I12" s="29">
         <f>COUNTIF(B12:H12,"Sí")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
-      <c r="B13" s="22" t="n"/>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="22" t="n"/>
-      <c r="G13" s="22" t="n"/>
-      <c r="H13" s="22" t="n"/>
-      <c r="I13" s="23">
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E13" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F13" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G13" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H13" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I13" s="29">
         <f>COUNTIF(B13:H13,"Sí")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="B14" s="22" t="n"/>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="22" t="n"/>
-      <c r="G14" s="22" t="n"/>
-      <c r="H14" s="22" t="n"/>
-      <c r="I14" s="23">
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E14" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F14" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G14" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H14" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I14" s="29">
         <f>COUNTIF(B14:H14,"Sí")</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>P9</t>
         </is>
       </c>
-      <c r="B15" s="22" t="n"/>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="22" t="n"/>
-      <c r="G15" s="22" t="n"/>
-      <c r="H15" s="22" t="n"/>
-      <c r="I15" s="23">
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G15" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H15" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I15" s="29">
         <f>COUNTIF(B15:H15,"Sí")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="B16" s="22" t="n"/>
-      <c r="C16" s="22" t="n"/>
-      <c r="D16" s="22" t="n"/>
-      <c r="E16" s="22" t="n"/>
-      <c r="F16" s="22" t="n"/>
-      <c r="G16" s="22" t="n"/>
-      <c r="H16" s="22" t="n"/>
-      <c r="I16" s="23">
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E16" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F16" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G16" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I16" s="29">
         <f>COUNTIF(B16:H16,"Sí")</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="B17" s="22" t="n"/>
-      <c r="C17" s="22" t="n"/>
-      <c r="D17" s="22" t="n"/>
-      <c r="E17" s="22" t="n"/>
-      <c r="F17" s="22" t="n"/>
-      <c r="G17" s="22" t="n"/>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="23">
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E17" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F17" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G17" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H17" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I17" s="29">
         <f>COUNTIF(B17:H17,"Sí")</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="B18" s="22" t="n"/>
-      <c r="C18" s="22" t="n"/>
-      <c r="D18" s="22" t="n"/>
-      <c r="E18" s="22" t="n"/>
-      <c r="F18" s="22" t="n"/>
-      <c r="G18" s="22" t="n"/>
-      <c r="H18" s="22" t="n"/>
-      <c r="I18" s="23">
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E18" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F18" s="29" t="inlineStr">
+        <is>
+          <t>Sí (parcial)</t>
+        </is>
+      </c>
+      <c r="G18" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H18" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I18" s="29">
         <f>COUNTIF(B18:H18,"Sí")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>P13</t>
         </is>
       </c>
-      <c r="B19" s="22" t="n"/>
-      <c r="C19" s="22" t="n"/>
-      <c r="D19" s="22" t="n"/>
-      <c r="E19" s="22" t="n"/>
-      <c r="F19" s="22" t="n"/>
-      <c r="G19" s="22" t="n"/>
-      <c r="H19" s="22" t="n"/>
-      <c r="I19" s="23">
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E19" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F19" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G19" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I19" s="29">
         <f>COUNTIF(B19:H19,"Sí")</f>
         <v/>
       </c>
@@ -1352,85 +1604,157 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>No (formulación estándar)</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>No administrada con la pregunta exacta; ofrece espontáneamente "es un monstruo... vino para quedarse" y "es mi amigo" en otros momentos.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>"Es una aplicación... que sirve para... está educada digitalmente a través de cosas que le fueron enseñando para que te pueda dar una respuesta." (instancia esforzada/honesta)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="18" t="n"/>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>No administrada con la formulación estándar; salta directo a casos de uso.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>"No me sale una definición, pero... está computado, una forma de decir una computadora, pero no es una computadora... te facilita la vida... mediante el prompt que vos le indiques." (instancia esforzada/honesta)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>P9</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>No administrada con la formulación estándar.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>P10</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>No (formulación estándar)</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>No administrada con la pregunta exacta; ofrece espontáneamente "es como mi secretaria" en otro momento.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>No administrada con la formulación estándar.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>No administrada como pregunta puntual, aunque ofrece definiciones extensas a lo largo de la entrevista.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>P13</t>
         </is>
       </c>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>"Una tecnología que aprende a partir de patrones de enormes cantidades de información... calculando qué palabras, imágenes o sonidos son más probables... por eso se equivoca, inventa datos o reproduce sesgos." Instancia más sofisticada del corpus.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="21" t="inlineStr">
@@ -1611,109 +1935,217 @@
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="18" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
-      <c r="E10" s="23">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>4 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>(ninguno estructuralmente nuevo -- refuerza objetivacion_imagen_concreta, anclaje_figura_humana, imaginario_inevitabilidad_tecnologica, imaginario_rol_docente_futuro, uso_iai_apoyo_administrativo)</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="25">
         <f>SUM($D$6:D10)</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
-      <c r="E11" s="23">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>5 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva (primera instancia clara)</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="25">
         <f>SUM($D$6:D11)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="18" t="n"/>
-      <c r="E12" s="23">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>6 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>adaptacion_saberes_previos (primera instancia), imaginario_desigualdad_estructural (primera instancia fuerte)</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="25">
         <f>SUM($D$6:D12)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="18" t="n"/>
-      <c r="D13" s="18" t="n"/>
-      <c r="E13" s="23">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>7 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>(refuerza varios; primera contra-instancia fuerte de imaginario_inevitabilidad_tecnologica e imaginario_rol_docente_futuro -- polaridad nueva, no código nuevo)</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="25">
         <f>SUM($D$6:D13)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="18" t="n"/>
-      <c r="E14" s="23">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>8 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>tension_autoria_impronta (primera instancia), eco_de_par_colega (2da instancia, inductivo reforzado), estrategia_deteccion_uso_estudiantil (candidato, primera mención)</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="25">
         <f>SUM($D$6:D14)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="23" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="23">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>9 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>estrategia_deteccion_uso_estudiantil (reforzado, método concreto) -- tension_autoria_impronta 2da instancia (más fuerte del corpus)</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="25">
         <f>SUM($D$6:D15)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="23">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>10 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>matiz de imaginario_desigualdad_estructural (acompañamiento familiar vs. clase social -- sub-dimensión, no código nuevo)</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="25">
         <f>SUM($D$6:D16)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="23" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="23">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>11 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>estrategia_deteccion_uso_estudiantil (reforzado con método concreto -- trampa textual)</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="25">
         <f>SUM($D$6:D17)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="23">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>12 (ajustar según tu orden real)</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>(informante elite; refuerza casi todos los códigos con alta densidad, sin categoría axial estructuralmente nueva)</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="25">
         <f>SUM($D$6:D18)</f>
         <v/>
       </c>
@@ -3246,17 +3678,17 @@
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>mito_estigma_pereza</t>
+          <t>estrategia_deteccion_uso_estudiantil</t>
         </is>
       </c>
       <c r="B9" s="29" t="inlineStr">
         <is>
-          <t>Referencia al estigma social/moral de que usar IA es "de vagos" o de facilismo -- distinto de imaginario_inevitabilidad_tecnologica (no es sobre si va a pasar) y de imaginario_rol_docente_futuro (no es sobre el rol futuro, es un juicio social presente).</t>
+          <t>Estrategias concretas que las docentes desarrollan para detectar cuando un estudiante entregó un trabajo generado por IA sin mediación propia (forense de estilo, trampas textuales, conocimiento del nivel real del alumno) -- distinto de competencia_critica_reflexiva (sobre la propia relación docente-IA) y de criterio_sentido_pedagogico (sobre diseño de propuestas).</t>
         </is>
       </c>
       <c r="C9" s="29" t="inlineStr">
         <is>
-          <t>Núcleo 4 (candidato -- en observación, n=1)</t>
+          <t>Núcleo 4 (candidato -- evidencia moderada, n=4: P3, P9, P10, P12)</t>
         </is>
       </c>
       <c r="D9" s="29" t="inlineStr">
@@ -3266,7 +3698,7 @@
       </c>
       <c r="E9" s="29" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>P10 (primera mención con método concreto; ecos previos en P3 y P9)</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4576,6 +5008,697 @@
       <c r="D74" s="18" t="n"/>
       <c r="E74" s="18" t="n"/>
     </row>
+    <row r="75">
+      <c r="A75" s="29" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B75" s="29" t="inlineStr">
+        <is>
+          <t>3/7</t>
+        </is>
+      </c>
+      <c r="C75" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta + imaginario_inevitabilidad_tecnologica</t>
+        </is>
+      </c>
+      <c r="D75" s="29" t="inlineStr">
+        <is>
+          <t>"es como un monstruo. Esto ya vino para quedarse y se va a quedar, creo. Y me fascina" [04:30]</t>
+        </is>
+      </c>
+      <c r="E75" s="29" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="29" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B76" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C76" s="29" t="inlineStr">
+        <is>
+          <t>anclaje_figura_humana</t>
+        </is>
+      </c>
+      <c r="D76" s="29" t="inlineStr">
+        <is>
+          <t>"el que más me gusta y es mi amigo es el ChatGPT... a veces pienso en un día esto me va a mandar a pasear" [04:59]-[05:26]</t>
+        </is>
+      </c>
+      <c r="E76" s="29" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="29" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B77" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C77" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D77" s="29" t="inlineStr">
+        <is>
+          <t>"no es usar el chat GPT y quedarnos con eso, sino saber qué preguntar y cómo preguntar" [04:00]-[04:30]; prioriza libros/papel antes de digital</t>
+        </is>
+      </c>
+      <c r="E77" s="29" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="29" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B78" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C78" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_rol_docente_futuro (negativo)</t>
+        </is>
+      </c>
+      <c r="D78" s="29" t="inlineStr">
+        <is>
+          <t>"siempre va a estar el docente aunque esté la inteligencia [muy] avanzada, siempre tenemos que intervenir para explicar" [15:48]-[16:18]</t>
+        </is>
+      </c>
+      <c r="E78" s="29" t="inlineStr">
+        <is>
+          <t>Rechaza narrativa de reemplazo</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="29" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B79" s="29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C79" s="29" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva (primera instancia clara)</t>
+        </is>
+      </c>
+      <c r="D79" s="29" t="inlineStr">
+        <is>
+          <t>"si es a libre uso... ahí no creo porque se limita todo a dame y ya está" [19:01]-[19:30]</t>
+        </is>
+      </c>
+      <c r="E79" s="29" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="29" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B80" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C80" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta</t>
+        </is>
+      </c>
+      <c r="D80" s="29" t="inlineStr">
+        <is>
+          <t>"es una aplicación... está educada digitalmente... para darte una respuesta" [10:32]-[11:43]</t>
+        </is>
+      </c>
+      <c r="E80" s="29" t="inlineStr">
+        <is>
+          <t>Instancia esforzada, similar a P2/P8</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="29" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B81" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C81" s="29" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D81" s="29" t="inlineStr">
+        <is>
+          <t>"el nuevo diseño curricular ya establece la educación digital como área transversal" [27:26]</t>
+        </is>
+      </c>
+      <c r="E81" s="29" t="inlineStr">
+        <is>
+          <t>Lo digital descrito como "algo impuesto"</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="29" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B82" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C82" s="29" t="inlineStr">
+        <is>
+          <t>adaptacion_saberes_previos + criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D82" s="29" t="inlineStr">
+        <is>
+          <t>"darle el texto y que me lo adecue con palabras más sencillas" para alumno con dificultades de integración [09:47]-[10:54]</t>
+        </is>
+      </c>
+      <c r="E82" s="29" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="29" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B83" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C83" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_desigualdad_estructural (primera instancia fuerte)</t>
+        </is>
+      </c>
+      <c r="D83" s="29" t="inlineStr">
+        <is>
+          <t>"en esos coles invierten en tecnología... acá no se está invirtiendo" — compara escuela actual (privada subvencionada, sin recursos) con anterior (privada de elite) [24:13]-[26:19]</t>
+        </is>
+      </c>
+      <c r="E83" s="29" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="29" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B84" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C84" s="29" t="inlineStr">
+        <is>
+          <t>potencia_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D84" s="29" t="inlineStr">
+        <is>
+          <t>Proyecto colaborativo 4 grados: IA estructuró actos de obra sobre Roald Dahl para coordinar escritura grupal [22:28]-[23:43]</t>
+        </is>
+      </c>
+      <c r="E84" s="29" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="29" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B85" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C85" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta</t>
+        </is>
+      </c>
+      <c r="D85" s="29" t="inlineStr">
+        <is>
+          <t>"está computado... una forma de decir una computadora, pero no es una computadora... te facilita la vida" [10:52]-[12:38]</t>
+        </is>
+      </c>
+      <c r="E85" s="29" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="29" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B86" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C86" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica (contra-instancia fuerte)</t>
+        </is>
+      </c>
+      <c r="D86" s="29" t="inlineStr">
+        <is>
+          <t>"no, no creo que cambie... para mí no va a cambiar nada [en 5 años]" — atribuye a falta de voluntad/resistencia docente, no a la tecnología [25:24]-[27:58]</t>
+        </is>
+      </c>
+      <c r="E86" s="29" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="29" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B87" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C87" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_rol_docente_futuro (contra-narrativa)</t>
+        </is>
+      </c>
+      <c r="D87" s="29" t="inlineStr">
+        <is>
+          <t>"no pienso que nos va a reemplazar... tenemos sentimientos" [18:09]-[18:52]</t>
+        </is>
+      </c>
+      <c r="E87" s="29" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="29" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B88" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C88" s="29" t="inlineStr">
+        <is>
+          <t>adaptacion_saberes_previos + criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D88" s="29" t="inlineStr">
+        <is>
+          <t>Actividad reparatoria armada con ChatGPT para alumno que no sabe leer/escribir [18:52]-[19:31]</t>
+        </is>
+      </c>
+      <c r="E88" s="29" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="29" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B89" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C89" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico + tension_autoria_impronta (primera instancia del corpus)</t>
+        </is>
+      </c>
+      <c r="D89" s="29" t="inlineStr">
+        <is>
+          <t>Carta de despedida: leyó versión de IA ("era perfecta") pero no la usó — "yo la quiero hacer, yo... lo que yo siento" [13:22]-[14:25]</t>
+        </is>
+      </c>
+      <c r="E89" s="29" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="29" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B90" s="29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C90" s="29" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D90" s="29" t="inlineStr">
+        <is>
+          <t>"es una herramienta más que no tiene que ocupar el 100%... tenemos que seguir enseñándoles a pensar" [18:05]-[19:28]</t>
+        </is>
+      </c>
+      <c r="E90" s="29" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="29" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B91" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C91" s="29" t="inlineStr">
+        <is>
+          <t>eco_de_par_colega (inductivo, 2ª instancia)</t>
+        </is>
+      </c>
+      <c r="D91" s="29" t="inlineStr">
+        <is>
+          <t>Amiga estudiante de abogacía relata que sus compañeros universitarios "no saben pensar... todo enseguida agarran el celular y ponen en la IA" [15:39]-[16:20]</t>
+        </is>
+      </c>
+      <c r="E91" s="29" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="29" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B92" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C92" s="29" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva</t>
+        </is>
+      </c>
+      <c r="D92" s="29" t="inlineStr">
+        <is>
+          <t>Coteja siempre en RAE; discute con quienes confían ciegamente en IA (anécdota "bandera" mayúscula/minúscula) [10:43]-[12:31]</t>
+        </is>
+      </c>
+      <c r="E92" s="29" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="29" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B93" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C93" s="29" t="inlineStr">
+        <is>
+          <t>tension_autoria_impronta (instancia más fuerte del corpus) + anclaje_figura_humana</t>
+        </is>
+      </c>
+      <c r="D93" s="29" t="inlineStr">
+        <is>
+          <t>"a mí me gusta que la planificación tenga mi impronta... si no me apropio, no lo doy bien" pero a la vez "es como mi secretaria" [13:46]-[15:43]</t>
+        </is>
+      </c>
+      <c r="E93" s="29" t="inlineStr">
+        <is>
+          <t>Alto uso y tensión de autoría coexisten</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="29" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B94" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C94" s="29" t="inlineStr">
+        <is>
+          <t>estrategia_deteccion_uso_estudiantil (inductivo candidato)</t>
+        </is>
+      </c>
+      <c r="D94" s="29" t="inlineStr">
+        <is>
+          <t>"sé cómo escribe ese alumno... si me trae todo con punto, coma, raya de diálogo bien puesta, entiendo que esto lo hiciste con la IA" [17:35]-[18:25]</t>
+        </is>
+      </c>
+      <c r="E94" s="29" t="inlineStr">
+        <is>
+          <t>Ver Log códigos inductivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="29" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B95" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C95" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_desigualdad_estructural</t>
+        </is>
+      </c>
+      <c r="D95" s="29" t="inlineStr">
+        <is>
+          <t>Referencia a película (sociedad dividida por acceso tecnológico) + Plan Sarmiento discontinuado [23:49]-[29:42]</t>
+        </is>
+      </c>
+      <c r="E95" s="29" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="29" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B96" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C96" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_desigualdad_estructural (matiz distinto)</t>
+        </is>
+      </c>
+      <c r="D96" s="29" t="inlineStr">
+        <is>
+          <t>"lo que más influye no es que sean pobres o de clase media... son los padres [presentes o no]" [18:58]-[20:45]</t>
+        </is>
+      </c>
+      <c r="E96" s="29" t="inlineStr">
+        <is>
+          <t>Sub-dimensión: acompañamiento familiar, no clase social</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="29" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B97" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C97" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D97" s="29" t="inlineStr">
+        <is>
+          <t>"si es realmente fructífero, si tiene sentido aplicar la tecnología o es solo para un adorno" [05:00]-[06:19]</t>
+        </is>
+      </c>
+      <c r="E97" s="29" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="29" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B98" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C98" s="29" t="inlineStr">
+        <is>
+          <t>estrategia_deteccion_uso_estudiantil (inductivo candidato, reforzado)</t>
+        </is>
+      </c>
+      <c r="D98" s="29" t="inlineStr">
+        <is>
+          <t>Colega insertó palabra oculta en texto blanco dentro de consigna; alumnos que copiaron de IA sin leer la repitieron sin darse cuenta [21:58]-[25:09]</t>
+        </is>
+      </c>
+      <c r="E98" s="29" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="29" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B99" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C99" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica</t>
+        </is>
+      </c>
+      <c r="D99" s="29" t="inlineStr">
+        <is>
+          <t>"es como que de repente digamos que no se use la energía eléctrica... ya está instalado... y es necesario" [26:11]-[27:58]</t>
+        </is>
+      </c>
+      <c r="E99" s="29" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="29" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B100" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C100" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta (instancia más sofisticada)</t>
+        </is>
+      </c>
+      <c r="D100" s="29" t="inlineStr">
+        <is>
+          <t>"tecnología que aprende a partir de patrones... calcula qué palabras/imágenes/sonidos son más probables... por eso se equivoca, inventa datos, reproduce sesgos" [10:26]-[12:23]</t>
+        </is>
+      </c>
+      <c r="E100" s="29" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="29" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B101" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C101" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica (escéptica de la narrativa)</t>
+        </is>
+      </c>
+      <c r="D101" s="29" t="inlineStr">
+        <is>
+          <t>"mi preocupación no radica tanto en la posibilidad tan generalizada que se dice... me preocupa el desconocimiento acerca de su funcionamiento" [15:47]-[16:47]</t>
+        </is>
+      </c>
+      <c r="E101" s="29" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="29" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B102" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C102" s="29" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional (variante crítica)</t>
+        </is>
+      </c>
+      <c r="D102" s="29" t="inlineStr">
+        <is>
+          <t>Capacitación situada reducida a "cómo dar un prompt en tono formal/coloquial"; cuestiona si hay "voluntad real" o "una banderita" [19:07]-[19:58]</t>
+        </is>
+      </c>
+      <c r="E102" s="29" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="29" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B103" s="29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C103" s="29" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva + potencia_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D103" s="29" t="inlineStr">
+        <is>
+          <t>"siempre y cuando estemos atentos a no tercerizar el proceso cognitivo"; riesgo cuando la IA "sustituye el esfuerzo de recordar, escribir, investigar" [21:26]-[23:48]</t>
+        </is>
+      </c>
+      <c r="E103" s="29" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Fix stray blank-row gap in Segmentos codificados sheet (P5-P13 were pushed down 38 rows)
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,6 +80,10 @@
       <i val="1"/>
       <color rgb="00808080"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="10">
@@ -138,7 +142,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -160,11 +164,12 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -245,6 +250,7 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4743,961 +4749,961 @@
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="18" t="n"/>
-      <c r="B37" s="18" t="n"/>
-      <c r="C37" s="18" t="n"/>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="18" t="n"/>
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B37" s="29" t="inlineStr">
+        <is>
+          <t>3/7</t>
+        </is>
+      </c>
+      <c r="C37" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta + imaginario_inevitabilidad_tecnologica</t>
+        </is>
+      </c>
+      <c r="D37" s="29" t="inlineStr">
+        <is>
+          <t>"es como un monstruo. Esto ya vino para quedarse y se va a quedar, creo. Y me fascina" [04:30]</t>
+        </is>
+      </c>
+      <c r="E37" s="29" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="18" t="n"/>
-      <c r="B38" s="18" t="n"/>
-      <c r="C38" s="18" t="n"/>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="18" t="n"/>
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C38" s="29" t="inlineStr">
+        <is>
+          <t>anclaje_figura_humana</t>
+        </is>
+      </c>
+      <c r="D38" s="29" t="inlineStr">
+        <is>
+          <t>"el que más me gusta y es mi amigo es el ChatGPT... a veces pienso en un día esto me va a mandar a pasear" [04:59]-[05:26]</t>
+        </is>
+      </c>
+      <c r="E38" s="29" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="18" t="n"/>
-      <c r="B39" s="18" t="n"/>
-      <c r="C39" s="18" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C39" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D39" s="29" t="inlineStr">
+        <is>
+          <t>"no es usar el chat GPT y quedarnos con eso, sino saber qué preguntar y cómo preguntar" [04:00]-[04:30]; prioriza libros/papel antes de digital</t>
+        </is>
+      </c>
+      <c r="E39" s="29" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="18" t="n"/>
-      <c r="B40" s="18" t="n"/>
-      <c r="C40" s="18" t="n"/>
-      <c r="D40" s="18" t="n"/>
-      <c r="E40" s="18" t="n"/>
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C40" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_rol_docente_futuro (negativo)</t>
+        </is>
+      </c>
+      <c r="D40" s="29" t="inlineStr">
+        <is>
+          <t>"siempre va a estar el docente aunque esté la inteligencia [muy] avanzada, siempre tenemos que intervenir para explicar" [15:48]-[16:18]</t>
+        </is>
+      </c>
+      <c r="E40" s="29" t="inlineStr">
+        <is>
+          <t>Rechaza narrativa de reemplazo</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="18" t="n"/>
-      <c r="B41" s="18" t="n"/>
-      <c r="C41" s="18" t="n"/>
-      <c r="D41" s="18" t="n"/>
-      <c r="E41" s="18" t="n"/>
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B41" s="29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C41" s="29" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva (primera instancia clara)</t>
+        </is>
+      </c>
+      <c r="D41" s="29" t="inlineStr">
+        <is>
+          <t>"si es a libre uso... ahí no creo porque se limita todo a dame y ya está" [19:01]-[19:30]</t>
+        </is>
+      </c>
+      <c r="E41" s="29" t="n"/>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="18" t="n"/>
-      <c r="B42" s="18" t="n"/>
-      <c r="C42" s="18" t="n"/>
-      <c r="D42" s="18" t="n"/>
-      <c r="E42" s="18" t="n"/>
+      <c r="A42" s="29" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B42" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta</t>
+        </is>
+      </c>
+      <c r="D42" s="29" t="inlineStr">
+        <is>
+          <t>"es una aplicación... está educada digitalmente... para darte una respuesta" [10:32]-[11:43]</t>
+        </is>
+      </c>
+      <c r="E42" s="29" t="inlineStr">
+        <is>
+          <t>Instancia esforzada, similar a P2/P8</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="18" t="n"/>
-      <c r="B43" s="18" t="n"/>
-      <c r="C43" s="18" t="n"/>
-      <c r="D43" s="18" t="n"/>
-      <c r="E43" s="18" t="n"/>
+      <c r="A43" s="29" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B43" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C43" s="29" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D43" s="29" t="inlineStr">
+        <is>
+          <t>"el nuevo diseño curricular ya establece la educación digital como área transversal" [27:26]</t>
+        </is>
+      </c>
+      <c r="E43" s="29" t="inlineStr">
+        <is>
+          <t>Lo digital descrito como "algo impuesto"</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="18" t="n"/>
-      <c r="B44" s="18" t="n"/>
-      <c r="C44" s="18" t="n"/>
-      <c r="D44" s="18" t="n"/>
-      <c r="E44" s="18" t="n"/>
+      <c r="A44" s="29" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B44" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C44" s="29" t="inlineStr">
+        <is>
+          <t>adaptacion_saberes_previos + criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D44" s="29" t="inlineStr">
+        <is>
+          <t>"darle el texto y que me lo adecue con palabras más sencillas" para alumno con dificultades de integración [09:47]-[10:54]</t>
+        </is>
+      </c>
+      <c r="E44" s="29" t="n"/>
     </row>
     <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="18" t="n"/>
-      <c r="B45" s="18" t="n"/>
-      <c r="C45" s="18" t="n"/>
-      <c r="D45" s="18" t="n"/>
-      <c r="E45" s="18" t="n"/>
+      <c r="A45" s="29" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B45" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C45" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_desigualdad_estructural (primera instancia fuerte)</t>
+        </is>
+      </c>
+      <c r="D45" s="29" t="inlineStr">
+        <is>
+          <t>"en esos coles invierten en tecnología... acá no se está invirtiendo" — compara escuela actual (privada subvencionada, sin recursos) con anterior (privada de elite) [24:13]-[26:19]</t>
+        </is>
+      </c>
+      <c r="E45" s="29" t="n"/>
     </row>
     <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="18" t="n"/>
-      <c r="B46" s="18" t="n"/>
-      <c r="C46" s="18" t="n"/>
-      <c r="D46" s="18" t="n"/>
-      <c r="E46" s="18" t="n"/>
+      <c r="A46" s="29" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B46" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C46" s="29" t="inlineStr">
+        <is>
+          <t>potencia_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D46" s="29" t="inlineStr">
+        <is>
+          <t>Proyecto colaborativo 4 grados: IA estructuró actos de obra sobre Roald Dahl para coordinar escritura grupal [22:28]-[23:43]</t>
+        </is>
+      </c>
+      <c r="E46" s="29" t="n"/>
     </row>
     <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="18" t="n"/>
-      <c r="B47" s="18" t="n"/>
-      <c r="C47" s="18" t="n"/>
-      <c r="D47" s="18" t="n"/>
-      <c r="E47" s="18" t="n"/>
+      <c r="A47" s="29" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B47" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C47" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta</t>
+        </is>
+      </c>
+      <c r="D47" s="29" t="inlineStr">
+        <is>
+          <t>"está computado... una forma de decir una computadora, pero no es una computadora... te facilita la vida" [10:52]-[12:38]</t>
+        </is>
+      </c>
+      <c r="E47" s="29" t="n"/>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="18" t="n"/>
-      <c r="B48" s="18" t="n"/>
-      <c r="C48" s="18" t="n"/>
-      <c r="D48" s="18" t="n"/>
-      <c r="E48" s="18" t="n"/>
+      <c r="A48" s="29" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B48" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C48" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica (contra-instancia fuerte)</t>
+        </is>
+      </c>
+      <c r="D48" s="29" t="inlineStr">
+        <is>
+          <t>"no, no creo que cambie... para mí no va a cambiar nada [en 5 años]" — atribuye a falta de voluntad/resistencia docente, no a la tecnología [25:24]-[27:58]</t>
+        </is>
+      </c>
+      <c r="E48" s="29" t="n"/>
     </row>
     <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="18" t="n"/>
-      <c r="B49" s="18" t="n"/>
-      <c r="C49" s="18" t="n"/>
-      <c r="D49" s="18" t="n"/>
-      <c r="E49" s="18" t="n"/>
+      <c r="A49" s="29" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B49" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_rol_docente_futuro (contra-narrativa)</t>
+        </is>
+      </c>
+      <c r="D49" s="29" t="inlineStr">
+        <is>
+          <t>"no pienso que nos va a reemplazar... tenemos sentimientos" [18:09]-[18:52]</t>
+        </is>
+      </c>
+      <c r="E49" s="29" t="n"/>
     </row>
     <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="18" t="n"/>
-      <c r="B50" s="18" t="n"/>
-      <c r="C50" s="18" t="n"/>
-      <c r="D50" s="18" t="n"/>
-      <c r="E50" s="18" t="n"/>
+      <c r="A50" s="29" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B50" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C50" s="29" t="inlineStr">
+        <is>
+          <t>adaptacion_saberes_previos + criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D50" s="29" t="inlineStr">
+        <is>
+          <t>Actividad reparatoria armada con ChatGPT para alumno que no sabe leer/escribir [18:52]-[19:31]</t>
+        </is>
+      </c>
+      <c r="E50" s="29" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="18" t="n"/>
-      <c r="B51" s="18" t="n"/>
-      <c r="C51" s="18" t="n"/>
-      <c r="D51" s="18" t="n"/>
-      <c r="E51" s="18" t="n"/>
+      <c r="A51" s="29" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B51" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C51" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico + tension_autoria_impronta (primera instancia del corpus)</t>
+        </is>
+      </c>
+      <c r="D51" s="29" t="inlineStr">
+        <is>
+          <t>Carta de despedida: leyó versión de IA ("era perfecta") pero no la usó — "yo la quiero hacer, yo... lo que yo siento" [13:22]-[14:25]</t>
+        </is>
+      </c>
+      <c r="E51" s="29" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="18" t="n"/>
-      <c r="B52" s="18" t="n"/>
-      <c r="C52" s="18" t="n"/>
-      <c r="D52" s="18" t="n"/>
-      <c r="E52" s="18" t="n"/>
+      <c r="A52" s="29" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B52" s="29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C52" s="29" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D52" s="29" t="inlineStr">
+        <is>
+          <t>"es una herramienta más que no tiene que ocupar el 100%... tenemos que seguir enseñándoles a pensar" [18:05]-[19:28]</t>
+        </is>
+      </c>
+      <c r="E52" s="29" t="n"/>
     </row>
     <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="18" t="n"/>
-      <c r="B53" s="18" t="n"/>
-      <c r="C53" s="18" t="n"/>
-      <c r="D53" s="18" t="n"/>
-      <c r="E53" s="18" t="n"/>
+      <c r="A53" s="29" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B53" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C53" s="29" t="inlineStr">
+        <is>
+          <t>eco_de_par_colega (inductivo, 2ª instancia)</t>
+        </is>
+      </c>
+      <c r="D53" s="29" t="inlineStr">
+        <is>
+          <t>Amiga estudiante de abogacía relata que sus compañeros universitarios "no saben pensar... todo enseguida agarran el celular y ponen en la IA" [15:39]-[16:20]</t>
+        </is>
+      </c>
+      <c r="E53" s="29" t="n"/>
     </row>
     <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="18" t="n"/>
-      <c r="B54" s="18" t="n"/>
-      <c r="C54" s="18" t="n"/>
-      <c r="D54" s="18" t="n"/>
-      <c r="E54" s="18" t="n"/>
+      <c r="A54" s="29" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B54" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C54" s="29" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva</t>
+        </is>
+      </c>
+      <c r="D54" s="29" t="inlineStr">
+        <is>
+          <t>Coteja siempre en RAE; discute con quienes confían ciegamente en IA (anécdota "bandera" mayúscula/minúscula) [10:43]-[12:31]</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="n"/>
     </row>
     <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="18" t="n"/>
-      <c r="B55" s="18" t="n"/>
-      <c r="C55" s="18" t="n"/>
-      <c r="D55" s="18" t="n"/>
-      <c r="E55" s="18" t="n"/>
+      <c r="A55" s="29" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B55" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C55" s="29" t="inlineStr">
+        <is>
+          <t>tension_autoria_impronta (instancia más fuerte del corpus) + anclaje_figura_humana</t>
+        </is>
+      </c>
+      <c r="D55" s="29" t="inlineStr">
+        <is>
+          <t>"a mí me gusta que la planificación tenga mi impronta... si no me apropio, no lo doy bien" pero a la vez "es como mi secretaria" [13:46]-[15:43]</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="inlineStr">
+        <is>
+          <t>Alto uso y tensión de autoría coexisten</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="18" t="n"/>
-      <c r="B56" s="18" t="n"/>
-      <c r="C56" s="18" t="n"/>
-      <c r="D56" s="18" t="n"/>
-      <c r="E56" s="18" t="n"/>
+      <c r="A56" s="29" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B56" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C56" s="29" t="inlineStr">
+        <is>
+          <t>estrategia_deteccion_uso_estudiantil (inductivo candidato)</t>
+        </is>
+      </c>
+      <c r="D56" s="29" t="inlineStr">
+        <is>
+          <t>"sé cómo escribe ese alumno... si me trae todo con punto, coma, raya de diálogo bien puesta, entiendo que esto lo hiciste con la IA" [17:35]-[18:25]</t>
+        </is>
+      </c>
+      <c r="E56" s="29" t="inlineStr">
+        <is>
+          <t>Ver Log códigos inductivos</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="18" t="n"/>
-      <c r="B57" s="18" t="n"/>
-      <c r="C57" s="18" t="n"/>
-      <c r="D57" s="18" t="n"/>
-      <c r="E57" s="18" t="n"/>
+      <c r="A57" s="29" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B57" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C57" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_desigualdad_estructural</t>
+        </is>
+      </c>
+      <c r="D57" s="29" t="inlineStr">
+        <is>
+          <t>Referencia a película (sociedad dividida por acceso tecnológico) + Plan Sarmiento discontinuado [23:49]-[29:42]</t>
+        </is>
+      </c>
+      <c r="E57" s="29" t="n"/>
     </row>
     <row r="58" ht="22" customHeight="1">
-      <c r="A58" s="18" t="n"/>
-      <c r="B58" s="18" t="n"/>
-      <c r="C58" s="18" t="n"/>
-      <c r="D58" s="18" t="n"/>
-      <c r="E58" s="18" t="n"/>
+      <c r="A58" s="29" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B58" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C58" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_desigualdad_estructural (matiz distinto)</t>
+        </is>
+      </c>
+      <c r="D58" s="29" t="inlineStr">
+        <is>
+          <t>"lo que más influye no es que sean pobres o de clase media... son los padres [presentes o no]" [18:58]-[20:45]</t>
+        </is>
+      </c>
+      <c r="E58" s="29" t="inlineStr">
+        <is>
+          <t>Sub-dimensión: acompañamiento familiar, no clase social</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="18" t="n"/>
-      <c r="B59" s="18" t="n"/>
-      <c r="C59" s="18" t="n"/>
-      <c r="D59" s="18" t="n"/>
-      <c r="E59" s="18" t="n"/>
+      <c r="A59" s="29" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B59" s="29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C59" s="29" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D59" s="29" t="inlineStr">
+        <is>
+          <t>"si es realmente fructífero, si tiene sentido aplicar la tecnología o es solo para un adorno" [05:00]-[06:19]</t>
+        </is>
+      </c>
+      <c r="E59" s="29" t="n"/>
     </row>
     <row r="60" ht="22" customHeight="1">
-      <c r="A60" s="18" t="n"/>
-      <c r="B60" s="18" t="n"/>
-      <c r="C60" s="18" t="n"/>
-      <c r="D60" s="18" t="n"/>
-      <c r="E60" s="18" t="n"/>
+      <c r="A60" s="29" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B60" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C60" s="29" t="inlineStr">
+        <is>
+          <t>estrategia_deteccion_uso_estudiantil (inductivo candidato, reforzado)</t>
+        </is>
+      </c>
+      <c r="D60" s="29" t="inlineStr">
+        <is>
+          <t>Colega insertó palabra oculta en texto blanco dentro de consigna; alumnos que copiaron de IA sin leer la repitieron sin darse cuenta [21:58]-[25:09]</t>
+        </is>
+      </c>
+      <c r="E60" s="29" t="n"/>
     </row>
     <row r="61" ht="22" customHeight="1">
-      <c r="A61" s="18" t="n"/>
-      <c r="B61" s="18" t="n"/>
-      <c r="C61" s="18" t="n"/>
-      <c r="D61" s="18" t="n"/>
-      <c r="E61" s="18" t="n"/>
+      <c r="A61" s="29" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B61" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C61" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica</t>
+        </is>
+      </c>
+      <c r="D61" s="29" t="inlineStr">
+        <is>
+          <t>"es como que de repente digamos que no se use la energía eléctrica... ya está instalado... y es necesario" [26:11]-[27:58]</t>
+        </is>
+      </c>
+      <c r="E61" s="29" t="n"/>
     </row>
     <row r="62" ht="22" customHeight="1">
-      <c r="A62" s="18" t="n"/>
-      <c r="B62" s="18" t="n"/>
-      <c r="C62" s="18" t="n"/>
-      <c r="D62" s="18" t="n"/>
-      <c r="E62" s="18" t="n"/>
+      <c r="A62" s="29" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B62" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C62" s="29" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta (instancia más sofisticada)</t>
+        </is>
+      </c>
+      <c r="D62" s="29" t="inlineStr">
+        <is>
+          <t>"tecnología que aprende a partir de patrones... calcula qué palabras/imágenes/sonidos son más probables... por eso se equivoca, inventa datos, reproduce sesgos" [10:26]-[12:23]</t>
+        </is>
+      </c>
+      <c r="E62" s="29" t="n"/>
     </row>
     <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="18" t="n"/>
-      <c r="B63" s="18" t="n"/>
-      <c r="C63" s="18" t="n"/>
-      <c r="D63" s="18" t="n"/>
-      <c r="E63" s="18" t="n"/>
+      <c r="A63" s="29" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B63" s="29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C63" s="29" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica (escéptica de la narrativa)</t>
+        </is>
+      </c>
+      <c r="D63" s="29" t="inlineStr">
+        <is>
+          <t>"mi preocupación no radica tanto en la posibilidad tan generalizada que se dice... me preocupa el desconocimiento acerca de su funcionamiento" [15:47]-[16:47]</t>
+        </is>
+      </c>
+      <c r="E63" s="29" t="n"/>
     </row>
     <row r="64" ht="22" customHeight="1">
-      <c r="A64" s="18" t="n"/>
-      <c r="B64" s="18" t="n"/>
-      <c r="C64" s="18" t="n"/>
-      <c r="D64" s="18" t="n"/>
-      <c r="E64" s="18" t="n"/>
+      <c r="A64" s="29" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B64" s="29" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C64" s="29" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional (variante crítica)</t>
+        </is>
+      </c>
+      <c r="D64" s="29" t="inlineStr">
+        <is>
+          <t>Capacitación situada reducida a "cómo dar un prompt en tono formal/coloquial"; cuestiona si hay "voluntad real" o "una banderita" [19:07]-[19:58]</t>
+        </is>
+      </c>
+      <c r="E64" s="29" t="n"/>
     </row>
     <row r="65" ht="22" customHeight="1">
-      <c r="A65" s="18" t="n"/>
-      <c r="B65" s="18" t="n"/>
-      <c r="C65" s="18" t="n"/>
-      <c r="D65" s="18" t="n"/>
-      <c r="E65" s="18" t="n"/>
+      <c r="A65" s="29" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B65" s="29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C65" s="29" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva + potencia_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D65" s="29" t="inlineStr">
+        <is>
+          <t>"siempre y cuando estemos atentos a no tercerizar el proceso cognitivo"; riesgo cuando la IA "sustituye el esfuerzo de recordar, escribir, investigar" [21:26]-[23:48]</t>
+        </is>
+      </c>
+      <c r="E65" s="29" t="n"/>
     </row>
     <row r="66" ht="22" customHeight="1">
-      <c r="A66" s="18" t="n"/>
-      <c r="B66" s="18" t="n"/>
-      <c r="C66" s="18" t="n"/>
-      <c r="D66" s="18" t="n"/>
-      <c r="E66" s="18" t="n"/>
+      <c r="A66" s="30" t="n"/>
+      <c r="B66" s="30" t="n"/>
+      <c r="C66" s="30" t="n"/>
+      <c r="D66" s="30" t="n"/>
+      <c r="E66" s="30" t="n"/>
     </row>
     <row r="67" ht="22" customHeight="1">
-      <c r="A67" s="18" t="n"/>
-      <c r="B67" s="18" t="n"/>
-      <c r="C67" s="18" t="n"/>
-      <c r="D67" s="18" t="n"/>
-      <c r="E67" s="18" t="n"/>
+      <c r="A67" s="30" t="n"/>
+      <c r="B67" s="30" t="n"/>
+      <c r="C67" s="30" t="n"/>
+      <c r="D67" s="30" t="n"/>
+      <c r="E67" s="30" t="n"/>
     </row>
     <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="18" t="n"/>
-      <c r="B68" s="18" t="n"/>
-      <c r="C68" s="18" t="n"/>
-      <c r="D68" s="18" t="n"/>
-      <c r="E68" s="18" t="n"/>
+      <c r="A68" s="30" t="n"/>
+      <c r="B68" s="30" t="n"/>
+      <c r="C68" s="30" t="n"/>
+      <c r="D68" s="30" t="n"/>
+      <c r="E68" s="30" t="n"/>
     </row>
     <row r="69" ht="22" customHeight="1">
-      <c r="A69" s="18" t="n"/>
-      <c r="B69" s="18" t="n"/>
-      <c r="C69" s="18" t="n"/>
-      <c r="D69" s="18" t="n"/>
-      <c r="E69" s="18" t="n"/>
+      <c r="A69" s="30" t="n"/>
+      <c r="B69" s="30" t="n"/>
+      <c r="C69" s="30" t="n"/>
+      <c r="D69" s="30" t="n"/>
+      <c r="E69" s="30" t="n"/>
     </row>
     <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="18" t="n"/>
-      <c r="B70" s="18" t="n"/>
-      <c r="C70" s="18" t="n"/>
-      <c r="D70" s="18" t="n"/>
-      <c r="E70" s="18" t="n"/>
+      <c r="A70" s="30" t="n"/>
+      <c r="B70" s="30" t="n"/>
+      <c r="C70" s="30" t="n"/>
+      <c r="D70" s="30" t="n"/>
+      <c r="E70" s="30" t="n"/>
     </row>
     <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="18" t="n"/>
-      <c r="B71" s="18" t="n"/>
-      <c r="C71" s="18" t="n"/>
-      <c r="D71" s="18" t="n"/>
-      <c r="E71" s="18" t="n"/>
+      <c r="A71" s="30" t="n"/>
+      <c r="B71" s="30" t="n"/>
+      <c r="C71" s="30" t="n"/>
+      <c r="D71" s="30" t="n"/>
+      <c r="E71" s="30" t="n"/>
     </row>
     <row r="72" ht="22" customHeight="1">
-      <c r="A72" s="18" t="n"/>
-      <c r="B72" s="18" t="n"/>
-      <c r="C72" s="18" t="n"/>
-      <c r="D72" s="18" t="n"/>
-      <c r="E72" s="18" t="n"/>
+      <c r="A72" s="30" t="n"/>
+      <c r="B72" s="30" t="n"/>
+      <c r="C72" s="30" t="n"/>
+      <c r="D72" s="30" t="n"/>
+      <c r="E72" s="30" t="n"/>
     </row>
     <row r="73" ht="22" customHeight="1">
-      <c r="A73" s="18" t="n"/>
-      <c r="B73" s="18" t="n"/>
-      <c r="C73" s="18" t="n"/>
-      <c r="D73" s="18" t="n"/>
-      <c r="E73" s="18" t="n"/>
+      <c r="A73" s="30" t="n"/>
+      <c r="B73" s="30" t="n"/>
+      <c r="C73" s="30" t="n"/>
+      <c r="D73" s="30" t="n"/>
+      <c r="E73" s="30" t="n"/>
     </row>
     <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="18" t="n"/>
-      <c r="B74" s="18" t="n"/>
-      <c r="C74" s="18" t="n"/>
-      <c r="D74" s="18" t="n"/>
-      <c r="E74" s="18" t="n"/>
+      <c r="A74" s="30" t="n"/>
+      <c r="B74" s="30" t="n"/>
+      <c r="C74" s="30" t="n"/>
+      <c r="D74" s="30" t="n"/>
+      <c r="E74" s="30" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="29" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B75" s="29" t="inlineStr">
-        <is>
-          <t>3/7</t>
-        </is>
-      </c>
-      <c r="C75" s="29" t="inlineStr">
-        <is>
-          <t>objetivacion_imagen_concreta + imaginario_inevitabilidad_tecnologica</t>
-        </is>
-      </c>
-      <c r="D75" s="29" t="inlineStr">
-        <is>
-          <t>"es como un monstruo. Esto ya vino para quedarse y se va a quedar, creo. Y me fascina" [04:30]</t>
-        </is>
-      </c>
-      <c r="E75" s="29" t="n"/>
+      <c r="A75" s="30" t="n"/>
+      <c r="B75" s="30" t="n"/>
+      <c r="C75" s="30" t="n"/>
+      <c r="D75" s="30" t="n"/>
+      <c r="E75" s="30" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="29" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B76" s="29" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C76" s="29" t="inlineStr">
-        <is>
-          <t>anclaje_figura_humana</t>
-        </is>
-      </c>
-      <c r="D76" s="29" t="inlineStr">
-        <is>
-          <t>"el que más me gusta y es mi amigo es el ChatGPT... a veces pienso en un día esto me va a mandar a pasear" [04:59]-[05:26]</t>
-        </is>
-      </c>
-      <c r="E76" s="29" t="n"/>
+      <c r="A76" s="30" t="n"/>
+      <c r="B76" s="30" t="n"/>
+      <c r="C76" s="30" t="n"/>
+      <c r="D76" s="30" t="n"/>
+      <c r="E76" s="30" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="29" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B77" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C77" s="29" t="inlineStr">
-        <is>
-          <t>criterio_sentido_pedagogico</t>
-        </is>
-      </c>
-      <c r="D77" s="29" t="inlineStr">
-        <is>
-          <t>"no es usar el chat GPT y quedarnos con eso, sino saber qué preguntar y cómo preguntar" [04:00]-[04:30]; prioriza libros/papel antes de digital</t>
-        </is>
-      </c>
-      <c r="E77" s="29" t="n"/>
+      <c r="A77" s="30" t="n"/>
+      <c r="B77" s="30" t="n"/>
+      <c r="C77" s="30" t="n"/>
+      <c r="D77" s="30" t="n"/>
+      <c r="E77" s="30" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="29" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="B78" s="29" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C78" s="29" t="inlineStr">
-        <is>
-          <t>imaginario_rol_docente_futuro (negativo)</t>
-        </is>
-      </c>
-      <c r="D78" s="29" t="inlineStr">
-        <is>
-          <t>"siempre va a estar el docente aunque esté la inteligencia [muy] avanzada, siempre tenemos que intervenir para explicar" [15:48]-[16:18]</t>
-        </is>
-      </c>
-      <c r="E78" s="29" t="inlineStr">
-        <is>
-          <t>Rechaza narrativa de reemplazo</t>
-        </is>
-      </c>
+      <c r="A78" s="30" t="n"/>
+      <c r="B78" s="30" t="n"/>
+      <c r="C78" s="30" t="n"/>
+      <c r="D78" s="30" t="n"/>
+      <c r="E78" s="30" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="29" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="B79" s="29" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C79" s="29" t="inlineStr">
-        <is>
-          <t>limita_integracion_sustantiva (primera instancia clara)</t>
-        </is>
-      </c>
-      <c r="D79" s="29" t="inlineStr">
-        <is>
-          <t>"si es a libre uso... ahí no creo porque se limita todo a dame y ya está" [19:01]-[19:30]</t>
-        </is>
-      </c>
-      <c r="E79" s="29" t="n"/>
+      <c r="A79" s="30" t="n"/>
+      <c r="B79" s="30" t="n"/>
+      <c r="C79" s="30" t="n"/>
+      <c r="D79" s="30" t="n"/>
+      <c r="E79" s="30" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="29" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="B80" s="29" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C80" s="29" t="inlineStr">
-        <is>
-          <t>objetivacion_imagen_concreta</t>
-        </is>
-      </c>
-      <c r="D80" s="29" t="inlineStr">
-        <is>
-          <t>"es una aplicación... está educada digitalmente... para darte una respuesta" [10:32]-[11:43]</t>
-        </is>
-      </c>
-      <c r="E80" s="29" t="inlineStr">
-        <is>
-          <t>Instancia esforzada, similar a P2/P8</t>
-        </is>
-      </c>
+      <c r="A80" s="30" t="n"/>
+      <c r="B80" s="30" t="n"/>
+      <c r="C80" s="30" t="n"/>
+      <c r="D80" s="30" t="n"/>
+      <c r="E80" s="30" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="29" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="B81" s="29" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C81" s="29" t="inlineStr">
-        <is>
-          <t>eco_discurso_institucional</t>
-        </is>
-      </c>
-      <c r="D81" s="29" t="inlineStr">
-        <is>
-          <t>"el nuevo diseño curricular ya establece la educación digital como área transversal" [27:26]</t>
-        </is>
-      </c>
-      <c r="E81" s="29" t="inlineStr">
-        <is>
-          <t>Lo digital descrito como "algo impuesto"</t>
-        </is>
-      </c>
+      <c r="A81" s="30" t="n"/>
+      <c r="B81" s="30" t="n"/>
+      <c r="C81" s="30" t="n"/>
+      <c r="D81" s="30" t="n"/>
+      <c r="E81" s="30" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="29" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B82" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C82" s="29" t="inlineStr">
-        <is>
-          <t>adaptacion_saberes_previos + criterio_contextual_grupo</t>
-        </is>
-      </c>
-      <c r="D82" s="29" t="inlineStr">
-        <is>
-          <t>"darle el texto y que me lo adecue con palabras más sencillas" para alumno con dificultades de integración [09:47]-[10:54]</t>
-        </is>
-      </c>
-      <c r="E82" s="29" t="n"/>
+      <c r="A82" s="30" t="n"/>
+      <c r="B82" s="30" t="n"/>
+      <c r="C82" s="30" t="n"/>
+      <c r="D82" s="30" t="n"/>
+      <c r="E82" s="30" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="29" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B83" s="29" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C83" s="29" t="inlineStr">
-        <is>
-          <t>imaginario_desigualdad_estructural (primera instancia fuerte)</t>
-        </is>
-      </c>
-      <c r="D83" s="29" t="inlineStr">
-        <is>
-          <t>"en esos coles invierten en tecnología... acá no se está invirtiendo" — compara escuela actual (privada subvencionada, sin recursos) con anterior (privada de elite) [24:13]-[26:19]</t>
-        </is>
-      </c>
-      <c r="E83" s="29" t="n"/>
+      <c r="A83" s="30" t="n"/>
+      <c r="B83" s="30" t="n"/>
+      <c r="C83" s="30" t="n"/>
+      <c r="D83" s="30" t="n"/>
+      <c r="E83" s="30" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="29" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="B84" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C84" s="29" t="inlineStr">
-        <is>
-          <t>potencia_integracion_sustantiva</t>
-        </is>
-      </c>
-      <c r="D84" s="29" t="inlineStr">
-        <is>
-          <t>Proyecto colaborativo 4 grados: IA estructuró actos de obra sobre Roald Dahl para coordinar escritura grupal [22:28]-[23:43]</t>
-        </is>
-      </c>
-      <c r="E84" s="29" t="n"/>
+      <c r="A84" s="30" t="n"/>
+      <c r="B84" s="30" t="n"/>
+      <c r="C84" s="30" t="n"/>
+      <c r="D84" s="30" t="n"/>
+      <c r="E84" s="30" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="29" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B85" s="29" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C85" s="29" t="inlineStr">
-        <is>
-          <t>objetivacion_imagen_concreta</t>
-        </is>
-      </c>
-      <c r="D85" s="29" t="inlineStr">
-        <is>
-          <t>"está computado... una forma de decir una computadora, pero no es una computadora... te facilita la vida" [10:52]-[12:38]</t>
-        </is>
-      </c>
-      <c r="E85" s="29" t="n"/>
+      <c r="A85" s="30" t="n"/>
+      <c r="B85" s="30" t="n"/>
+      <c r="C85" s="30" t="n"/>
+      <c r="D85" s="30" t="n"/>
+      <c r="E85" s="30" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="29" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B86" s="29" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C86" s="29" t="inlineStr">
-        <is>
-          <t>imaginario_inevitabilidad_tecnologica (contra-instancia fuerte)</t>
-        </is>
-      </c>
-      <c r="D86" s="29" t="inlineStr">
-        <is>
-          <t>"no, no creo que cambie... para mí no va a cambiar nada [en 5 años]" — atribuye a falta de voluntad/resistencia docente, no a la tecnología [25:24]-[27:58]</t>
-        </is>
-      </c>
-      <c r="E86" s="29" t="n"/>
+      <c r="A86" s="30" t="n"/>
+      <c r="B86" s="30" t="n"/>
+      <c r="C86" s="30" t="n"/>
+      <c r="D86" s="30" t="n"/>
+      <c r="E86" s="30" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="29" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B87" s="29" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C87" s="29" t="inlineStr">
-        <is>
-          <t>imaginario_rol_docente_futuro (contra-narrativa)</t>
-        </is>
-      </c>
-      <c r="D87" s="29" t="inlineStr">
-        <is>
-          <t>"no pienso que nos va a reemplazar... tenemos sentimientos" [18:09]-[18:52]</t>
-        </is>
-      </c>
-      <c r="E87" s="29" t="n"/>
+      <c r="A87" s="30" t="n"/>
+      <c r="B87" s="30" t="n"/>
+      <c r="C87" s="30" t="n"/>
+      <c r="D87" s="30" t="n"/>
+      <c r="E87" s="30" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="29" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="B88" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C88" s="29" t="inlineStr">
-        <is>
-          <t>adaptacion_saberes_previos + criterio_contextual_grupo</t>
-        </is>
-      </c>
-      <c r="D88" s="29" t="inlineStr">
-        <is>
-          <t>Actividad reparatoria armada con ChatGPT para alumno que no sabe leer/escribir [18:52]-[19:31]</t>
-        </is>
-      </c>
-      <c r="E88" s="29" t="n"/>
+      <c r="A88" s="30" t="n"/>
+      <c r="B88" s="30" t="n"/>
+      <c r="C88" s="30" t="n"/>
+      <c r="D88" s="30" t="n"/>
+      <c r="E88" s="30" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="29" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="B89" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C89" s="29" t="inlineStr">
-        <is>
-          <t>criterio_sentido_pedagogico + tension_autoria_impronta (primera instancia del corpus)</t>
-        </is>
-      </c>
-      <c r="D89" s="29" t="inlineStr">
-        <is>
-          <t>Carta de despedida: leyó versión de IA ("era perfecta") pero no la usó — "yo la quiero hacer, yo... lo que yo siento" [13:22]-[14:25]</t>
-        </is>
-      </c>
-      <c r="E89" s="29" t="n"/>
+      <c r="A89" s="30" t="n"/>
+      <c r="B89" s="30" t="n"/>
+      <c r="C89" s="30" t="n"/>
+      <c r="D89" s="30" t="n"/>
+      <c r="E89" s="30" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="29" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="B90" s="29" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C90" s="29" t="inlineStr">
-        <is>
-          <t>limita_integracion_sustantiva</t>
-        </is>
-      </c>
-      <c r="D90" s="29" t="inlineStr">
-        <is>
-          <t>"es una herramienta más que no tiene que ocupar el 100%... tenemos que seguir enseñándoles a pensar" [18:05]-[19:28]</t>
-        </is>
-      </c>
-      <c r="E90" s="29" t="n"/>
+      <c r="A90" s="30" t="n"/>
+      <c r="B90" s="30" t="n"/>
+      <c r="C90" s="30" t="n"/>
+      <c r="D90" s="30" t="n"/>
+      <c r="E90" s="30" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="29" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="B91" s="29" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C91" s="29" t="inlineStr">
-        <is>
-          <t>eco_de_par_colega (inductivo, 2ª instancia)</t>
-        </is>
-      </c>
-      <c r="D91" s="29" t="inlineStr">
-        <is>
-          <t>Amiga estudiante de abogacía relata que sus compañeros universitarios "no saben pensar... todo enseguida agarran el celular y ponen en la IA" [15:39]-[16:20]</t>
-        </is>
-      </c>
-      <c r="E91" s="29" t="n"/>
+      <c r="A91" s="30" t="n"/>
+      <c r="B91" s="30" t="n"/>
+      <c r="C91" s="30" t="n"/>
+      <c r="D91" s="30" t="n"/>
+      <c r="E91" s="30" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="29" t="inlineStr">
-        <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="B92" s="29" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C92" s="29" t="inlineStr">
-        <is>
-          <t>competencia_critica_reflexiva</t>
-        </is>
-      </c>
-      <c r="D92" s="29" t="inlineStr">
-        <is>
-          <t>Coteja siempre en RAE; discute con quienes confían ciegamente en IA (anécdota "bandera" mayúscula/minúscula) [10:43]-[12:31]</t>
-        </is>
-      </c>
-      <c r="E92" s="29" t="n"/>
+      <c r="A92" s="30" t="n"/>
+      <c r="B92" s="30" t="n"/>
+      <c r="C92" s="30" t="n"/>
+      <c r="D92" s="30" t="n"/>
+      <c r="E92" s="30" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="29" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="B93" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C93" s="29" t="inlineStr">
-        <is>
-          <t>tension_autoria_impronta (instancia más fuerte del corpus) + anclaje_figura_humana</t>
-        </is>
-      </c>
-      <c r="D93" s="29" t="inlineStr">
-        <is>
-          <t>"a mí me gusta que la planificación tenga mi impronta... si no me apropio, no lo doy bien" pero a la vez "es como mi secretaria" [13:46]-[15:43]</t>
-        </is>
-      </c>
-      <c r="E93" s="29" t="inlineStr">
-        <is>
-          <t>Alto uso y tensión de autoría coexisten</t>
-        </is>
-      </c>
+      <c r="A93" s="30" t="n"/>
+      <c r="B93" s="30" t="n"/>
+      <c r="C93" s="30" t="n"/>
+      <c r="D93" s="30" t="n"/>
+      <c r="E93" s="30" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="29" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="B94" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C94" s="29" t="inlineStr">
-        <is>
-          <t>estrategia_deteccion_uso_estudiantil (inductivo candidato)</t>
-        </is>
-      </c>
-      <c r="D94" s="29" t="inlineStr">
-        <is>
-          <t>"sé cómo escribe ese alumno... si me trae todo con punto, coma, raya de diálogo bien puesta, entiendo que esto lo hiciste con la IA" [17:35]-[18:25]</t>
-        </is>
-      </c>
-      <c r="E94" s="29" t="inlineStr">
-        <is>
-          <t>Ver Log códigos inductivos</t>
-        </is>
-      </c>
+      <c r="A94" s="30" t="n"/>
+      <c r="B94" s="30" t="n"/>
+      <c r="C94" s="30" t="n"/>
+      <c r="D94" s="30" t="n"/>
+      <c r="E94" s="30" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="29" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="B95" s="29" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C95" s="29" t="inlineStr">
-        <is>
-          <t>imaginario_desigualdad_estructural</t>
-        </is>
-      </c>
-      <c r="D95" s="29" t="inlineStr">
-        <is>
-          <t>Referencia a película (sociedad dividida por acceso tecnológico) + Plan Sarmiento discontinuado [23:49]-[29:42]</t>
-        </is>
-      </c>
-      <c r="E95" s="29" t="n"/>
+      <c r="A95" s="30" t="n"/>
+      <c r="B95" s="30" t="n"/>
+      <c r="C95" s="30" t="n"/>
+      <c r="D95" s="30" t="n"/>
+      <c r="E95" s="30" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="29" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="B96" s="29" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C96" s="29" t="inlineStr">
-        <is>
-          <t>imaginario_desigualdad_estructural (matiz distinto)</t>
-        </is>
-      </c>
-      <c r="D96" s="29" t="inlineStr">
-        <is>
-          <t>"lo que más influye no es que sean pobres o de clase media... son los padres [presentes o no]" [18:58]-[20:45]</t>
-        </is>
-      </c>
-      <c r="E96" s="29" t="inlineStr">
-        <is>
-          <t>Sub-dimensión: acompañamiento familiar, no clase social</t>
-        </is>
-      </c>
+      <c r="A96" s="30" t="n"/>
+      <c r="B96" s="30" t="n"/>
+      <c r="C96" s="30" t="n"/>
+      <c r="D96" s="30" t="n"/>
+      <c r="E96" s="30" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="29" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="B97" s="29" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C97" s="29" t="inlineStr">
-        <is>
-          <t>criterio_sentido_pedagogico</t>
-        </is>
-      </c>
-      <c r="D97" s="29" t="inlineStr">
-        <is>
-          <t>"si es realmente fructífero, si tiene sentido aplicar la tecnología o es solo para un adorno" [05:00]-[06:19]</t>
-        </is>
-      </c>
-      <c r="E97" s="29" t="n"/>
+      <c r="A97" s="30" t="n"/>
+      <c r="B97" s="30" t="n"/>
+      <c r="C97" s="30" t="n"/>
+      <c r="D97" s="30" t="n"/>
+      <c r="E97" s="30" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="29" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="B98" s="29" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C98" s="29" t="inlineStr">
-        <is>
-          <t>estrategia_deteccion_uso_estudiantil (inductivo candidato, reforzado)</t>
-        </is>
-      </c>
-      <c r="D98" s="29" t="inlineStr">
-        <is>
-          <t>Colega insertó palabra oculta en texto blanco dentro de consigna; alumnos que copiaron de IA sin leer la repitieron sin darse cuenta [21:58]-[25:09]</t>
-        </is>
-      </c>
-      <c r="E98" s="29" t="n"/>
+      <c r="A98" s="30" t="n"/>
+      <c r="B98" s="30" t="n"/>
+      <c r="C98" s="30" t="n"/>
+      <c r="D98" s="30" t="n"/>
+      <c r="E98" s="30" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="29" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="B99" s="29" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C99" s="29" t="inlineStr">
-        <is>
-          <t>imaginario_inevitabilidad_tecnologica</t>
-        </is>
-      </c>
-      <c r="D99" s="29" t="inlineStr">
-        <is>
-          <t>"es como que de repente digamos que no se use la energía eléctrica... ya está instalado... y es necesario" [26:11]-[27:58]</t>
-        </is>
-      </c>
-      <c r="E99" s="29" t="n"/>
+      <c r="A99" s="30" t="n"/>
+      <c r="B99" s="30" t="n"/>
+      <c r="C99" s="30" t="n"/>
+      <c r="D99" s="30" t="n"/>
+      <c r="E99" s="30" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="29" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="B100" s="29" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C100" s="29" t="inlineStr">
-        <is>
-          <t>objetivacion_imagen_concreta (instancia más sofisticada)</t>
-        </is>
-      </c>
-      <c r="D100" s="29" t="inlineStr">
-        <is>
-          <t>"tecnología que aprende a partir de patrones... calcula qué palabras/imágenes/sonidos son más probables... por eso se equivoca, inventa datos, reproduce sesgos" [10:26]-[12:23]</t>
-        </is>
-      </c>
-      <c r="E100" s="29" t="n"/>
+      <c r="A100" s="30" t="n"/>
+      <c r="B100" s="30" t="n"/>
+      <c r="C100" s="30" t="n"/>
+      <c r="D100" s="30" t="n"/>
+      <c r="E100" s="30" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="29" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="B101" s="29" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C101" s="29" t="inlineStr">
-        <is>
-          <t>imaginario_inevitabilidad_tecnologica (escéptica de la narrativa)</t>
-        </is>
-      </c>
-      <c r="D101" s="29" t="inlineStr">
-        <is>
-          <t>"mi preocupación no radica tanto en la posibilidad tan generalizada que se dice... me preocupa el desconocimiento acerca de su funcionamiento" [15:47]-[16:47]</t>
-        </is>
-      </c>
-      <c r="E101" s="29" t="n"/>
+      <c r="A101" s="30" t="n"/>
+      <c r="B101" s="30" t="n"/>
+      <c r="C101" s="30" t="n"/>
+      <c r="D101" s="30" t="n"/>
+      <c r="E101" s="30" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="29" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="B102" s="29" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C102" s="29" t="inlineStr">
-        <is>
-          <t>eco_discurso_institucional (variante crítica)</t>
-        </is>
-      </c>
-      <c r="D102" s="29" t="inlineStr">
-        <is>
-          <t>Capacitación situada reducida a "cómo dar un prompt en tono formal/coloquial"; cuestiona si hay "voluntad real" o "una banderita" [19:07]-[19:58]</t>
-        </is>
-      </c>
-      <c r="E102" s="29" t="n"/>
+      <c r="A102" s="30" t="n"/>
+      <c r="B102" s="30" t="n"/>
+      <c r="C102" s="30" t="n"/>
+      <c r="D102" s="30" t="n"/>
+      <c r="E102" s="30" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="29" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="B103" s="29" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C103" s="29" t="inlineStr">
-        <is>
-          <t>limita_integracion_sustantiva + potencia_integracion_sustantiva</t>
-        </is>
-      </c>
-      <c r="D103" s="29" t="inlineStr">
-        <is>
-          <t>"siempre y cuando estemos atentos a no tercerizar el proceso cognitivo"; riesgo cuando la IA "sustituye el esfuerzo de recordar, escribir, investigar" [21:26]-[23:48]</t>
-        </is>
-      </c>
-      <c r="E103" s="29" t="n"/>
+      <c r="A103" s="30" t="n"/>
+      <c r="B103" s="30" t="n"/>
+      <c r="C103" s="30" t="n"/>
+      <c r="D103" s="30" t="n"/>
+      <c r="E103" s="30" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Code P15 against codebook v1 — corpus now 14/15 (P1-P13 + P15)
No structurally new axial category. Reinforces limita_integracion_sustantiva,
criterio_sentido_pedagogico, competencia_critica_reflexiva, eco_discurso_institucional;
rich counter-instance for imaginario_rol_docente_futuro (explicit rejection of
teacher-replacement narrative); relativizing nuance for
imaginario_inevitabilidad_tecnologica. One n=1 inductive candidate logged, not
promoted (etica_regulacion_autonomia_infantil). Consistent with the theoretical
saturation signal already reported after P10-P13. Capítulo 3 §3.3 updated to
14/15 transcripts. Reflexivity: prior relationship with this participant flagged
explicitly as unconfirmed, not assumed. Raw transcript stored local-only
(gitignored), per standing data-privacy convention.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -1466,13 +1466,41 @@
           <t>P15</t>
         </is>
       </c>
-      <c r="B21" s="22" t="n"/>
-      <c r="C21" s="22" t="n"/>
-      <c r="D21" s="22" t="n"/>
-      <c r="E21" s="22" t="n"/>
-      <c r="F21" s="22" t="n"/>
-      <c r="G21" s="22" t="n"/>
-      <c r="H21" s="22" t="n"/>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="inlineStr">
+        <is>
+          <t>Sí (parcial -- corte de conexión durante la respuesta, retomada)</t>
+        </is>
+      </c>
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H21" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="I21" s="23">
         <f>COUNTIF(B21:H21,"Sí")</f>
         <v/>
@@ -1777,8 +1805,16 @@
           <t>P15</t>
         </is>
       </c>
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="18" t="n"/>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Sí (reformulada: "explicale a un colega" en vez de "a alguien")</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>"Es un asistente, uno lo puede utilizar como asistente de trabajo para uno o para los chicos." Framing funcional (anclaje_figura_humana), no metáfora espontánea libre.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2157,12 +2193,24 @@
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="23" t="n">
-        <v>13</v>
-      </c>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>13 (orden real -- P14 aún no recibida)</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>(ninguna categoría axial estructuralmente nueva -- refuerza fuertemente limita_integracion_sustantiva, criterio_sentido_pedagogico, competencia_critica_reflexiva, eco_discurso_institucional; contra-instancia rica de imaginario_rol_docente_futuro; matiz relativizador de imaginario_inevitabilidad_tecnologica; candidato inductivo n=1 sin promover (etica_regulacion_autonomia_infantil))</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="E19" s="23">
         <f>SUM($D$6:D19)</f>
         <v/>
@@ -2398,9 +2446,21 @@
           <t>P15</t>
         </is>
       </c>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>A CONFIRMAR CON LA INVESTIGADORA -- no se infiere de la transcripción</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5440,116 +5500,436 @@
       <c r="E65" s="29" t="n"/>
     </row>
     <row r="66" ht="22" customHeight="1">
-      <c r="A66" s="30" t="n"/>
-      <c r="B66" s="30" t="n"/>
-      <c r="C66" s="30" t="n"/>
-      <c r="D66" s="30" t="n"/>
-      <c r="E66" s="30" t="n"/>
+      <c r="A66" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B66" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C66" s="30" t="inlineStr">
+        <is>
+          <t>competencia_tecnica_declarada</t>
+        </is>
+      </c>
+      <c r="D66" s="30" t="inlineStr">
+        <is>
+          <t>"alto gusto y altos conocimientos... mi tesis tiene que ver con la educación del teatro en entornos digitales" [02:53-03:59]</t>
+        </is>
+      </c>
+      <c r="E66" s="30" t="inlineStr">
+        <is>
+          <t>Perfil de alta competencia declarada, con formación de posgrado propia en el cruce arte-tecnología</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="22" customHeight="1">
-      <c r="A67" s="30" t="n"/>
-      <c r="B67" s="30" t="n"/>
-      <c r="C67" s="30" t="n"/>
-      <c r="D67" s="30" t="n"/>
-      <c r="E67" s="30" t="n"/>
+      <c r="A67" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B67" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C67" s="30" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D67" s="30" t="inlineStr">
+        <is>
+          <t>"nos fijábamos que tuviese que ver con el texto... que no fuera una estética sesgada que viene estructurada desde la IA" [05:46]</t>
+        </is>
+      </c>
+      <c r="E67" s="30" t="inlineStr">
+        <is>
+          <t>Vigilancia activa del sesgo estético por defecto de la IA frente al contenido curricular (teatro griego)</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="30" t="n"/>
-      <c r="B68" s="30" t="n"/>
-      <c r="C68" s="30" t="n"/>
-      <c r="D68" s="30" t="n"/>
-      <c r="E68" s="30" t="n"/>
+      <c r="A68" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B68" s="30" t="inlineStr">
+        <is>
+          <t>3 (ancla)</t>
+        </is>
+      </c>
+      <c r="C68" s="30" t="inlineStr">
+        <is>
+          <t>anclaje_figura_humana</t>
+        </is>
+      </c>
+      <c r="D68" s="30" t="inlineStr">
+        <is>
+          <t>"es un asistente... de trabajo para uno o para los chicos" [06:32-06:58]</t>
+        </is>
+      </c>
+      <c r="E68" s="30" t="inlineStr">
+        <is>
+          <t>Respuesta a la pregunta ancla, reformulada como "explicale a un colega" -- framing funcional</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="22" customHeight="1">
-      <c r="A69" s="30" t="n"/>
-      <c r="B69" s="30" t="n"/>
-      <c r="C69" s="30" t="n"/>
-      <c r="D69" s="30" t="n"/>
-      <c r="E69" s="30" t="n"/>
+      <c r="A69" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B69" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C69" s="30" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva, limita_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D69" s="30" t="inlineStr">
+        <is>
+          <t>"las planificaciones terminan siendo todas muy parecidas... si uno no interviene, si las clases son siempre iguales" [06:58-07:25]</t>
+        </is>
+      </c>
+      <c r="E69" s="30" t="inlineStr">
+        <is>
+          <t>Riesgo de homogeneización si se usa sin criterio propio</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="30" t="n"/>
-      <c r="B70" s="30" t="n"/>
-      <c r="C70" s="30" t="n"/>
-      <c r="D70" s="30" t="n"/>
-      <c r="E70" s="30" t="n"/>
+      <c r="A70" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B70" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C70" s="30" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D70" s="30" t="inlineStr">
+        <is>
+          <t>"mientras más conocimiento de la didáctica, del área específica, de la evaluación, [mejor] las prácticas con esa herramienta" [07:25-07:45]</t>
+        </is>
+      </c>
+      <c r="E70" s="30" t="inlineStr">
+        <is>
+          <t>Conocimiento disciplinar/pedagógico condiciona la calidad del uso, no la competencia digital en sí</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="30" t="n"/>
-      <c r="B71" s="30" t="n"/>
-      <c r="C71" s="30" t="n"/>
-      <c r="D71" s="30" t="n"/>
-      <c r="E71" s="30" t="n"/>
+      <c r="A71" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B71" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C71" s="30" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva, eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D71" s="30" t="inlineStr">
+        <is>
+          <t>"trabajar con los chicos mucho el pensamiento crítico" [08:05-08:33]</t>
+        </is>
+      </c>
+      <c r="E71" s="30" t="inlineStr">
+        <is>
+          <t>Eco del marcador "pensamiento crítico"/4C, Guía CABA p.5</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="22" customHeight="1">
-      <c r="A72" s="30" t="n"/>
-      <c r="B72" s="30" t="n"/>
-      <c r="C72" s="30" t="n"/>
-      <c r="D72" s="30" t="n"/>
-      <c r="E72" s="30" t="n"/>
+      <c r="A72" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B72" s="30" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C72" s="30" t="inlineStr">
+        <is>
+          <t>criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D72" s="30" t="inlineStr">
+        <is>
+          <t>"con los más chicos no lo trabajé porque trabajo en primer ciclo" [08:33-09:01]</t>
+        </is>
+      </c>
+      <c r="E72" s="30" t="inlineStr">
+        <is>
+          <t>Criterio etario explícito</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="22" customHeight="1">
-      <c r="A73" s="30" t="n"/>
-      <c r="B73" s="30" t="n"/>
-      <c r="C73" s="30" t="n"/>
-      <c r="D73" s="30" t="n"/>
-      <c r="E73" s="30" t="n"/>
+      <c r="A73" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B73" s="30" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C73" s="30" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D73" s="30" t="inlineStr">
+        <is>
+          <t>"doble estructura, uno que ellos creen un cuento, después que la IA cree otro... si no, la creación queda sesgada" [09:01-09:30]</t>
+        </is>
+      </c>
+      <c r="E73" s="30" t="inlineStr">
+        <is>
+          <t>Diseño didáctico anti-sustitución -- buena cita candidata para Cap. 4</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="30" t="n"/>
-      <c r="B74" s="30" t="n"/>
-      <c r="C74" s="30" t="n"/>
-      <c r="D74" s="30" t="n"/>
-      <c r="E74" s="30" t="n"/>
+      <c r="A74" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B74" s="30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C74" s="30" t="inlineStr">
+        <is>
+          <t>etica_regulacion_autonomia_infantil (inductivo candidato, n=1)</t>
+        </is>
+      </c>
+      <c r="D74" s="30" t="inlineStr">
+        <is>
+          <t>"deberíamos tener... algún tipo de ética de uso y de regulación... hay todo un proceso de autonomía de los nenes que hay que trabajar" [11:08-11:53]</t>
+        </is>
+      </c>
+      <c r="E74" s="30" t="inlineStr">
+        <is>
+          <t>No calza limpio en ningún código existente -- centrado en autonomía infantil como condición previa, no solo regulación general. n=1, no promover todavía</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="30" t="n"/>
-      <c r="B75" s="30" t="n"/>
-      <c r="C75" s="30" t="n"/>
-      <c r="D75" s="30" t="n"/>
-      <c r="E75" s="30" t="n"/>
+      <c r="A75" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B75" s="30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C75" s="30" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva, anclaje_tecnologia_previa</t>
+        </is>
+      </c>
+      <c r="D75" s="30" t="inlineStr">
+        <is>
+          <t>"ya ni siquiera el Google, le preguntan [a la IA]" [11:53-12:23]</t>
+        </is>
+      </c>
+      <c r="E75" s="30" t="inlineStr">
+        <is>
+          <t>Instancia de anclaje_tecnologia_previa (contraste con buscador), referida al uso familiar/doméstico, no al propio uso docente</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="30" t="n"/>
-      <c r="B76" s="30" t="n"/>
-      <c r="C76" s="30" t="n"/>
-      <c r="D76" s="30" t="n"/>
-      <c r="E76" s="30" t="n"/>
+      <c r="A76" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B76" s="30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D76" s="30" t="inlineStr">
+        <is>
+          <t>"mientras más herramientas hay, [más] formación docente haya, el uso... va a ser más claro" [13:49-14:18]</t>
+        </is>
+      </c>
+      <c r="E76" s="30" t="inlineStr">
+        <is>
+          <t>Eco del marcador "formación continua"</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="30" t="n"/>
-      <c r="B77" s="30" t="n"/>
-      <c r="C77" s="30" t="n"/>
-      <c r="D77" s="30" t="n"/>
-      <c r="E77" s="30" t="n"/>
+      <c r="A77" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B77" s="30" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva, criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D77" s="30" t="inlineStr">
+        <is>
+          <t>"no tiene una experticia... si el docente no lo pensó, no está... la IA lo puede ayudar, orientar u ordenar" [16:34-17:32]</t>
+        </is>
+      </c>
+      <c r="E77" s="30" t="inlineStr">
+        <is>
+          <t>El aprendizaje significativo depende del diseño docente, no de la IA en sí -- cita fuerte y clara, candidata para Cap. 4/Discusión</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="30" t="n"/>
-      <c r="B78" s="30" t="n"/>
-      <c r="C78" s="30" t="n"/>
-      <c r="D78" s="30" t="n"/>
-      <c r="E78" s="30" t="n"/>
+      <c r="A78" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B78" s="30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C78" s="30" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica (matizado)</t>
+        </is>
+      </c>
+      <c r="D78" s="30" t="inlineStr">
+        <is>
+          <t>"por ahí ahora es una moda, después será un elemento más" [18:29-19:16]</t>
+        </is>
+      </c>
+      <c r="E78" s="30" t="inlineStr">
+        <is>
+          <t>Desdramatiza la inevitabilidad, normaliza sin narrativa de ruptura</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="30" t="n"/>
-      <c r="B79" s="30" t="n"/>
-      <c r="C79" s="30" t="n"/>
-      <c r="D79" s="30" t="n"/>
-      <c r="E79" s="30" t="n"/>
+      <c r="A79" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B79" s="30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C79" s="30" t="inlineStr">
+        <is>
+          <t>imaginario_rol_docente_futuro (contra-instancia)</t>
+        </is>
+      </c>
+      <c r="D79" s="30" t="inlineStr">
+        <is>
+          <t>"no creo que [reemplacen al docente]... el niño tiene otras características de socializar... está más centrada para los adultos" [19:16-19:56]</t>
+        </is>
+      </c>
+      <c r="E79" s="30" t="inlineStr">
+        <is>
+          <t>Rechazo explícito de la narrativa de reemplazo docente/automatización</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="30" t="n"/>
-      <c r="B80" s="30" t="n"/>
-      <c r="C80" s="30" t="n"/>
-      <c r="D80" s="30" t="n"/>
-      <c r="E80" s="30" t="n"/>
+      <c r="A80" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B80" s="30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C80" s="30" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D80" s="30" t="inlineStr">
+        <is>
+          <t>"pienso en un código, una ética, una legislación... la capacidad crítica" [20:28-21:23]</t>
+        </is>
+      </c>
+      <c r="E80" s="30" t="inlineStr">
+        <is>
+          <t>Eco fuerte de "uso responsable, ético y crítico" + "pensamiento crítico"</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="30" t="n"/>
-      <c r="B81" s="30" t="n"/>
-      <c r="C81" s="30" t="n"/>
-      <c r="D81" s="30" t="n"/>
-      <c r="E81" s="30" t="n"/>
+      <c r="A81" s="30" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B81" s="30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C81" s="30" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva</t>
+        </is>
+      </c>
+      <c r="D81" s="30" t="inlineStr">
+        <is>
+          <t>"se hackea a sí misma sin querer... es un modo de enseñar la ética" [21:23-21:53]</t>
+        </is>
+      </c>
+      <c r="E81" s="30" t="inlineStr">
+        <is>
+          <t>Errores/alucinaciones de la IA como oportunidad pedagógica -- eco parcial del marcador "sesgos/alucinaciones"</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="30" t="n"/>

</xml_diff>

<commit_message>
Resolve P15 validation questions: reflexividad and inductive candidate
Researcher confirms: (1) Eugenia (P15) has an indirect institutional
link (student of the thesis director, not of the researcher) --
logged as a distinct subcategory from P8/P10/P13's direct link;
(2) etica_regulacion_autonomia_infantil (n=1) not promoted to a new
code, absorbed into eco_discurso_institucional with an explicit note
preserved in the codebook so the nuance isn't lost.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -2448,7 +2448,7 @@
       </c>
       <c r="B20" s="18" t="inlineStr">
         <is>
-          <t>A CONFIRMAR CON LA INVESTIGADORA -- no se infiere de la transcripción</t>
+          <t>Indirecto: no fue alumna de la investigadora, pero sí fue estudiante de su directora de tesis (vínculo institucional vía dirección de tesis, distinto del vínculo directo de P8/P10/P13)</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -5728,7 +5728,7 @@
       </c>
       <c r="C74" s="30" t="inlineStr">
         <is>
-          <t>etica_regulacion_autonomia_infantil (inductivo candidato, n=1)</t>
+          <t>eco_discurso_institucional</t>
         </is>
       </c>
       <c r="D74" s="30" t="inlineStr">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>No calza limpio en ningún código existente -- centrado en autonomía infantil como condición previa, no solo regulación general. n=1, no promover todavía</t>
+          <t>No calza limpio en los marcadores institucionales previos -- centrado en autonomía infantil como condición previa al uso de cualquier tecnología. Propuesto como candidato inductivo separado (etica_regulacion_autonomia_infantil); la investigadora decidió (2026-08-05) absorberlo acá en vez de crear código nuevo, con nota conservada en la definición del código en codebook_v0_manual.md. Reevaluar si el matiz reaparece con volumen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close the corpus: code P1 and P14, complete N=15/15
Corrects a pre-existing off-by-one in the corpus count (P1 had never
actually been coded despite earlier docs implying 14 cases; the real
prior count was 13: P2-P13 + P15). Notable finding: P1 breaks the
prior total absence of eco_imaginario_mercantil_mediatico with an
explicit media-sourced echo -- changes that finding's framing in Cap.
4 from "substantive absence" to "rare but present." criterio_sentido_
pedagogico confirmed as the corpus's highest-frequency code (11/15).
Theoretical saturation proposed as reached in Cap. 3 §3.7, pending the
researcher's final confirmation. Full detail and five open validation
questions in codificacion_P1_P14_cierre_corpus.md.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -878,13 +878,41 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n"/>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="22" t="n"/>
-      <c r="F7" s="22" t="n"/>
-      <c r="G7" s="22" t="n"/>
-      <c r="H7" s="22" t="n"/>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>Sí (implícita, sin pregunta formal "explicá a alguien")</t>
+        </is>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>Sí (parcial -- vía áreas curriculares, no framing explícito de "aprendizaje significativo")</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>No (no se preguntó escenario a 5-10 años explícito, aunque sí habilidades futuras)</t>
+        </is>
+      </c>
       <c r="I7" s="23">
         <f>COUNTIF(B7:H7,"Sí")</f>
         <v/>
@@ -1448,13 +1476,41 @@
           <t>P14</t>
         </is>
       </c>
-      <c r="B20" s="22" t="n"/>
-      <c r="C20" s="22" t="n"/>
-      <c r="D20" s="22" t="n"/>
-      <c r="E20" s="22" t="n"/>
-      <c r="F20" s="22" t="n"/>
-      <c r="G20" s="22" t="n"/>
-      <c r="H20" s="22" t="n"/>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>Sí (ancla privilegiada administrada)</t>
+        </is>
+      </c>
+      <c r="E20" s="22" t="inlineStr">
+        <is>
+          <t>Sí (implícito, dentro de la respuesta de aprendizaje significativo, no bloque separado)</t>
+        </is>
+      </c>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G20" s="22" t="inlineStr">
+        <is>
+          <t>Sí (parcial -- vía flyers/proyectos, no framing explícito de "propuesta didáctica")</t>
+        </is>
+      </c>
+      <c r="H20" s="22" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="I20" s="23">
         <f>COUNTIF(B20:H20,"Sí")</f>
         <v/>
@@ -1583,8 +1639,16 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="18" t="n"/>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>No administrada (no se formuló la pregunta "explicale a alguien qué es")</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Sin metáfora espontánea clara -- describe la IA en términos de uso/riesgo ("puede volverse como un vicio"), no de definición.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="25" t="inlineStr">
@@ -1796,8 +1860,16 @@
           <t>P14</t>
         </is>
       </c>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>"Es una plataforma que genera texto y a la vez comprende texto... puede generar imágenes, puede generar videos. Genera recursos a partir de una solicitud que le hace el usuario." Definición técnico-funcional, mismo registro que P13 (instancia sofisticada), no metáfora.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="21" t="inlineStr">
@@ -2217,24 +2289,48 @@
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="23" t="n">
-        <v>14</v>
-      </c>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>14 (orden real)</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>eco_imaginario_mercantil_mediatico (PRIMERA INSTANCIA del corpus completo -- rompe el 0/14 previo), preocupacion_recursos_materiales_infraestructura (refuerzo fuerte, inductivo ya existente)</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="E20" s="23">
         <f>SUM($D$6:D20)</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="23" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" s="18" t="n"/>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="18" t="n"/>
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>15 (orden real -- cierre de corpus)</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>(ninguna categoría axial estructuralmente nueva -- refuerza fuertemente criterio_sentido_pedagogico, criterio_contextual_grupo, limita_integracion_sustantiva, eco_discurso_institucional, imaginario_inevitabilidad_tecnologica, imaginario_rol_docente_futuro)</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="E21" s="23">
         <f>SUM($D$6:D21)</f>
         <v/>
@@ -2306,9 +2402,21 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n"/>
-      <c r="C6" s="18" t="n"/>
-      <c r="D6" s="18" t="n"/>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="50" customHeight="1">
       <c r="A7" s="21" t="inlineStr">
@@ -2436,9 +2544,21 @@
           <t>P14</t>
         </is>
       </c>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="50" customHeight="1">
       <c r="A20" s="21" t="inlineStr">
@@ -5932,158 +6052,598 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="30" t="n"/>
-      <c r="B82" s="30" t="n"/>
-      <c r="C82" s="30" t="n"/>
-      <c r="D82" s="30" t="n"/>
-      <c r="E82" s="30" t="n"/>
+      <c r="A82" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B82" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C82" s="30" t="inlineStr">
+        <is>
+          <t>competencia_tecnica_declarada</t>
+        </is>
+      </c>
+      <c r="D82" s="30" t="inlineStr">
+        <is>
+          <t>"Estoy como en un nivel medio. Hace poco empecé a usar la inteligencia artificial"</t>
+        </is>
+      </c>
+      <c r="E82" s="30" t="inlineStr">
+        <is>
+          <t>Autoevaluación media, en contraste con perfiles "elite" del corpus (P8,P13,P15)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="30" t="n"/>
-      <c r="B83" s="30" t="n"/>
-      <c r="C83" s="30" t="n"/>
-      <c r="D83" s="30" t="n"/>
-      <c r="E83" s="30" t="n"/>
+      <c r="A83" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B83" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C83" s="30" t="inlineStr">
+        <is>
+          <t>preocupacion_recursos_materiales_infraestructura (inductivo)</t>
+        </is>
+      </c>
+      <c r="D83" s="30" t="inlineStr">
+        <is>
+          <t>"Hay muchas barreras cada vez que quiero usar algo... si quiero grabar sonido, ¿dónde lo guardamos?"</t>
+        </is>
+      </c>
+      <c r="E83" s="30" t="inlineStr">
+        <is>
+          <t>Refuerza el código inductivo de P2 -- barreras concretas de infraestructura/tiempo, no de formación</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="30" t="n"/>
-      <c r="B84" s="30" t="n"/>
-      <c r="C84" s="30" t="n"/>
-      <c r="D84" s="30" t="n"/>
-      <c r="E84" s="30" t="n"/>
+      <c r="A84" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B84" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C84" s="30" t="inlineStr">
+        <is>
+          <t>eco_de_par_colega (inductivo)</t>
+        </is>
+      </c>
+      <c r="D84" s="30" t="inlineStr">
+        <is>
+          <t>"Sé que en una de mis escuelas, una docente con la facilitadora hicieron una investigación con los chicos... pero no tengo muchos más detalles"</t>
+        </is>
+      </c>
+      <c r="E84" s="30" t="inlineStr">
+        <is>
+          <t>Tercera instancia del corpus (con P3, P9) -- representación mediada por un tercero</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="30" t="n"/>
-      <c r="B85" s="30" t="n"/>
-      <c r="C85" s="30" t="n"/>
-      <c r="D85" s="30" t="n"/>
-      <c r="E85" s="30" t="n"/>
+      <c r="A85" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B85" s="30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C85" s="30" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D85" s="30" t="inlineStr">
+        <is>
+          <t>"Siento que puede volverse como un vicio... Me preocupa que quienes recién se están formando no desarrollen habilidades propias"</t>
+        </is>
+      </c>
+      <c r="E85" s="30" t="inlineStr">
+        <is>
+          <t>Instancia clara -- preocupación por desarrollo de habilidades propias, no solo del resultado</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="30" t="n"/>
-      <c r="B86" s="30" t="n"/>
-      <c r="C86" s="30" t="n"/>
-      <c r="D86" s="30" t="n"/>
-      <c r="E86" s="30" t="n"/>
+      <c r="A86" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B86" s="30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C86" s="30" t="inlineStr">
+        <is>
+          <t>eco_imaginario_mercantil_mediatico (inductivo, ya en codebook)</t>
+        </is>
+      </c>
+      <c r="D86" s="30" t="inlineStr">
+        <is>
+          <t>"Vi en la tele que empresas como OpenAI están vinculadas con temas armamentísticos, con la guerra en Irán, y eso me genera desconfianza"</t>
+        </is>
+      </c>
+      <c r="E86" s="30" t="inlineStr">
+        <is>
+          <t>PRIMERA INSTANCIA del corpus completo (0/14 -&gt; 1/15) -- eco mediático explícito, fuente declarada ("vi en la tele")</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="30" t="n"/>
-      <c r="B87" s="30" t="n"/>
-      <c r="C87" s="30" t="n"/>
-      <c r="D87" s="30" t="n"/>
-      <c r="E87" s="30" t="n"/>
+      <c r="A87" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B87" s="30" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C87" s="30" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D87" s="30" t="inlineStr">
+        <is>
+          <t>"[Un alumno] la trajo hecha con IA. Y yo pensé: ¿qué gracia tiene?... se trata de aprender, no de que lo haga otro"</t>
+        </is>
+      </c>
+      <c r="E87" s="30" t="inlineStr">
+        <is>
+          <t>Cita candidata fuerte para Cap. 4 -- objeto: creación artística/blues</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="30" t="n"/>
-      <c r="B88" s="30" t="n"/>
-      <c r="C88" s="30" t="n"/>
-      <c r="D88" s="30" t="n"/>
-      <c r="E88" s="30" t="n"/>
+      <c r="A88" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B88" s="30" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C88" s="30" t="inlineStr">
+        <is>
+          <t>criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D88" s="30" t="inlineStr">
+        <is>
+          <t>"En los grados más chicos no le veo mucha aplicación. Los chicos tienen que aprender lo básico, no delegarlo a la IA"</t>
+        </is>
+      </c>
+      <c r="E88" s="30" t="inlineStr">
+        <is>
+          <t>Criterio etario explícito</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="30" t="n"/>
-      <c r="B89" s="30" t="n"/>
-      <c r="C89" s="30" t="n"/>
-      <c r="D89" s="30" t="n"/>
-      <c r="E89" s="30" t="n"/>
+      <c r="A89" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B89" s="30" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C89" s="30" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D89" s="30" t="inlineStr">
+        <is>
+          <t>"La consigna no estaba pensada para trabajar con IA. Por eso le pedí que tomara alguna idea, pero que hiciera su propio trabajo"</t>
+        </is>
+      </c>
+      <c r="E89" s="30" t="inlineStr">
+        <is>
+          <t>Reflexión retrospectiva sobre diseño de consigna, post-episodio del blues</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="30" t="n"/>
-      <c r="B90" s="30" t="n"/>
-      <c r="C90" s="30" t="n"/>
-      <c r="D90" s="30" t="n"/>
-      <c r="E90" s="30" t="n"/>
+      <c r="A90" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B90" s="30" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C90" s="30" t="inlineStr">
+        <is>
+          <t>uso_iai_apoyo_administrativo</t>
+        </is>
+      </c>
+      <c r="D90" s="30" t="inlineStr">
+        <is>
+          <t>"El director me pidió un proyecto para el concurso Cooperar, y armé algo con ayuda de la IA"</t>
+        </is>
+      </c>
+      <c r="E90" s="30" t="inlineStr">
+        <is>
+          <t>Uso institucional/de gestión (presentación a concurso), no estrictamente administrativo puro -- caso híbrido</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="30" t="n"/>
-      <c r="B91" s="30" t="n"/>
-      <c r="C91" s="30" t="n"/>
-      <c r="D91" s="30" t="n"/>
-      <c r="E91" s="30" t="n"/>
+      <c r="A91" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B91" s="30" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C91" s="30" t="inlineStr">
+        <is>
+          <t>tension_autoria_impronta</t>
+        </is>
+      </c>
+      <c r="D91" s="30" t="inlineStr">
+        <is>
+          <t>"Le pedía una idea a la IA, y después la modificaba en base a lo que yo quería. Pero me servía la estructura"</t>
+        </is>
+      </c>
+      <c r="E91" s="30" t="inlineStr">
+        <is>
+          <t>Patrón de uso: retiene autoría propia, usa la IA solo como andamiaje/estructura</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="30" t="n"/>
-      <c r="B92" s="30" t="n"/>
-      <c r="C92" s="30" t="n"/>
-      <c r="D92" s="30" t="n"/>
-      <c r="E92" s="30" t="n"/>
+      <c r="A92" s="30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B92" s="30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C92" s="30" t="inlineStr">
+        <is>
+          <t>competencia_critica_reflexiva</t>
+        </is>
+      </c>
+      <c r="D92" s="30" t="inlineStr">
+        <is>
+          <t>"Primero, conocerla. Usarla uno mismo... tener clara la intención de uso"</t>
+        </is>
+      </c>
+      <c r="E92" s="30" t="inlineStr">
+        <is>
+          <t>Sobre las competencias que debería tener un docente</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="30" t="n"/>
-      <c r="B93" s="30" t="n"/>
-      <c r="C93" s="30" t="n"/>
-      <c r="D93" s="30" t="n"/>
-      <c r="E93" s="30" t="n"/>
+      <c r="A93" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B93" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C93" s="30" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D93" s="30" t="inlineStr">
+        <is>
+          <t>"Tengo en cuenta que el recurso no sea el foco de la clase, sino más bien un recurso... el foco tiene que ser el contenido"</t>
+        </is>
+      </c>
+      <c r="E93" s="30" t="inlineStr">
+        <is>
+          <t>Instancia muy clara y explícita -- principio general de su práctica</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="30" t="n"/>
-      <c r="B94" s="30" t="n"/>
-      <c r="C94" s="30" t="n"/>
-      <c r="D94" s="30" t="n"/>
-      <c r="E94" s="30" t="n"/>
+      <c r="A94" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B94" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C94" s="30" t="inlineStr">
+        <is>
+          <t>criterio_sentido_pedagogico</t>
+        </is>
+      </c>
+      <c r="D94" s="30" t="inlineStr">
+        <is>
+          <t>"No utilizo plataformas de programación para programar, sino para trabajar conceptos de programación"</t>
+        </is>
+      </c>
+      <c r="E94" s="30" t="inlineStr">
+        <is>
+          <t>Segunda instancia, mismo principio aplicado a un caso concreto (Scratch/Makeymakey)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="30" t="n"/>
-      <c r="B95" s="30" t="n"/>
-      <c r="C95" s="30" t="n"/>
-      <c r="D95" s="30" t="n"/>
-      <c r="E95" s="30" t="n"/>
+      <c r="A95" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B95" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C95" s="30" t="inlineStr">
+        <is>
+          <t>criterio_contextual_grupo</t>
+        </is>
+      </c>
+      <c r="D95" s="30" t="inlineStr">
+        <is>
+          <t>"Hay alumnos que pueden arrastrar muy bien bloques... y hay otros alumnos que no, entonces lograr que todos vayan a la par... lleva tiempo"</t>
+        </is>
+      </c>
+      <c r="E95" s="30" t="inlineStr">
+        <is>
+          <t>Heterogeneidad de competencias digitales dentro del grupo como variable de planificación</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="30" t="n"/>
-      <c r="B96" s="30" t="n"/>
-      <c r="C96" s="30" t="n"/>
-      <c r="D96" s="30" t="n"/>
-      <c r="E96" s="30" t="n"/>
+      <c r="A96" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B96" s="30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C96" s="30" t="inlineStr">
+        <is>
+          <t>objetivacion_imagen_concreta</t>
+        </is>
+      </c>
+      <c r="D96" s="30" t="inlineStr">
+        <is>
+          <t>"Es una plataforma que genera texto y a la vez comprende texto... genera recursos a partir de una solicitud que le hace el usuario"</t>
+        </is>
+      </c>
+      <c r="E96" s="30" t="inlineStr">
+        <is>
+          <t>Ancla privilegiada (Bloque 3, P1) -- definición técnico-funcional, mismo registro que P13</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="30" t="n"/>
-      <c r="B97" s="30" t="n"/>
-      <c r="C97" s="30" t="n"/>
-      <c r="D97" s="30" t="n"/>
-      <c r="E97" s="30" t="n"/>
+      <c r="A97" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B97" s="30" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C97" s="30" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D97" s="30" t="inlineStr">
+        <is>
+          <t>"Ver si hay sesgos, ver el tema del prompteo..."</t>
+        </is>
+      </c>
+      <c r="E97" s="30" t="inlineStr">
+        <is>
+          <t>Eco directo del marcador "sesgos/alucinaciones" (Guía Nación p.8, glosario Guía CABA)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="30" t="n"/>
-      <c r="B98" s="30" t="n"/>
-      <c r="C98" s="30" t="n"/>
-      <c r="D98" s="30" t="n"/>
-      <c r="E98" s="30" t="n"/>
+      <c r="A98" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B98" s="30" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C98" s="30" t="inlineStr">
+        <is>
+          <t>eco_discurso_institucional</t>
+        </is>
+      </c>
+      <c r="D98" s="30" t="inlineStr">
+        <is>
+          <t>"Dejarle el legado al estudiante de que tiene que ser crítico, reflexivo... con esto de los sesgos"</t>
+        </is>
+      </c>
+      <c r="E98" s="30" t="inlineStr">
+        <is>
+          <t>Eco de "pensamiento crítico"/4C (Guía CABA p.5)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="30" t="n"/>
-      <c r="B99" s="30" t="n"/>
-      <c r="C99" s="30" t="n"/>
-      <c r="D99" s="30" t="n"/>
-      <c r="E99" s="30" t="n"/>
+      <c r="A99" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B99" s="30" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C99" s="30" t="inlineStr">
+        <is>
+          <t>limita_integracion_sustantiva</t>
+        </is>
+      </c>
+      <c r="D99" s="30" t="inlineStr">
+        <is>
+          <t>"Delega mucho trabajo cognitivo cuando se adapta demasiado a estas plataformas... qué perdemos cuando delegamos tanto"</t>
+        </is>
+      </c>
+      <c r="E99" s="30" t="inlineStr">
+        <is>
+          <t>Preocupación explícita por costo cognitivo de la delegación</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="30" t="n"/>
-      <c r="B100" s="30" t="n"/>
-      <c r="C100" s="30" t="n"/>
-      <c r="D100" s="30" t="n"/>
-      <c r="E100" s="30" t="n"/>
+      <c r="A100" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B100" s="30" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C100" s="30" t="inlineStr">
+        <is>
+          <t>uso_iai_apoyo_administrativo</t>
+        </is>
+      </c>
+      <c r="D100" s="30" t="inlineStr">
+        <is>
+          <t>"También las he usado... para generar flyers sobre proyectos"</t>
+        </is>
+      </c>
+      <c r="E100" s="30" t="inlineStr">
+        <is>
+          <t>Uso instrumental/promocional, distinto del uso pedagógico directo con alumnos</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="30" t="n"/>
-      <c r="B101" s="30" t="n"/>
-      <c r="C101" s="30" t="n"/>
-      <c r="D101" s="30" t="n"/>
-      <c r="E101" s="30" t="n"/>
+      <c r="A101" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B101" s="30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C101" s="30" t="inlineStr">
+        <is>
+          <t>imaginario_inevitabilidad_tecnologica</t>
+        </is>
+      </c>
+      <c r="D101" s="30" t="inlineStr">
+        <is>
+          <t>"Va a ser competencia de todos... va a ser necesario que tengamos competencias digitales... porque te acelera mucho los procesos"</t>
+        </is>
+      </c>
+      <c r="E101" s="30" t="inlineStr">
+        <is>
+          <t>Instancia afirmativa clara -- se suma a P4,P5,P12</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="30" t="n"/>
-      <c r="B102" s="30" t="n"/>
-      <c r="C102" s="30" t="n"/>
-      <c r="D102" s="30" t="n"/>
-      <c r="E102" s="30" t="n"/>
+      <c r="A102" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B102" s="30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C102" s="30" t="inlineStr">
+        <is>
+          <t>imaginario_rol_docente_futuro</t>
+        </is>
+      </c>
+      <c r="D102" s="30" t="inlineStr">
+        <is>
+          <t>"Un docente que sabe utilizarla y aprovecharla bien va a lograr resultados mucho más rápido que un docente que no"</t>
+        </is>
+      </c>
+      <c r="E102" s="30" t="inlineStr">
+        <is>
+          <t>Visión de diferenciación futura entre docentes según manejo de IA</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="30" t="n"/>
-      <c r="B103" s="30" t="n"/>
-      <c r="C103" s="30" t="n"/>
-      <c r="D103" s="30" t="n"/>
-      <c r="E103" s="30" t="n"/>
+      <c r="A103" s="30" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B103" s="30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C103" s="30" t="inlineStr">
+        <is>
+          <t>tension_autoria_impronta</t>
+        </is>
+      </c>
+      <c r="D103" s="30" t="inlineStr">
+        <is>
+          <t>"Me genera cierto ruido delegarle todo a la IA y perder lo genuino de lo humano... revalorar el trabajo humano y lo auténtico humano"</t>
+        </is>
+      </c>
+      <c r="E103" s="30" t="inlineStr">
+        <is>
+          <t>Registro generalizado/filosófico, no autorreferido a su propia planificación -- instancia más blanda que P9/P10, marcar la diferencia de registro</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Add producto/proceso vs. aprendizaje-articulado inductive code pair
Formalizes the researcher's observation that concrete AI-usage
examples across the corpus describe what was made or how it was used,
but never what students actually learned. Reread the full 15-interview
corpus: ejemplo_centrado_producto_proceso appears in 5/15 (7 examples,
all product/process-only); its mirror aprendizaje_explicitado_en_ejemplo
found 0/15 on active search. Unplanned finding along the way: P12
supplies observed evidence that learning did NOT occur (students who
copied from AI repeated a hidden trap word without noticing) -- doesn't
fit either new code, flagged separately as the strongest evidence in
either direction anywhere in the corpus.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -2723,7 +2723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2824,6 +2824,40 @@
       <c r="D7" s="10" t="inlineStr">
         <is>
           <t>"No sé si sabe con qué grupo estoy trabajando"</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ejemplo_centrado_producto_proceso (inductivo, 2026-08-07)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Al describir un ejemplo concreto de uso de IAG, la docente articula qué se produjo o cómo se usó la herramienta, pero no qué comprendieron/lograron los estudiantes.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hay un ejemplo concreto narrado (no opinión general) y el relato se agota en producto/proceso, sin mención de aprendizaje observado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>aprendizaje_explicitado_en_ejemplo (inductivo, 2026-08-07 -- espejo del anterior)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>La docente sí articula, en un ejemplo concreto, qué comprendió/logró el estudiante como resultado del uso de IAG.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Buscar activamente (regla anti-forcing). Resultado relectura 2026-08-07: 0/15.</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4041,6 +4075,60 @@
       <c r="C31" s="18" t="n"/>
       <c r="D31" s="18" t="n"/>
       <c r="E31" s="18" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ejemplo_centrado_producto_proceso</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Ejemplo concreto de uso de IAG donde se articula producto/proceso pero no aprendizaje del estudiante.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Núcleo 2 (cruza con Núcleo 5)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Observación de la investigadora sobre la matriz de patrones; relectura corpus completo: 5/15 (P1,P3x2,P7,P8,P15x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>aprendizaje_explicitado_en_ejemplo</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Código espejo -- la docente sí articula un resultado de aprendizaje del estudiante en un ejemplo concreto.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Núcleo 2</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Búsqueda activa en relectura corpus completo: 0/15 -- ausencia real, buscada, no solo constatada por omisión</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4057,7 +4145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6645,6 +6733,222 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>ejemplo_centrado_producto_proceso</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>"El director me pidió un proyecto para el concurso Cooperar... una narrativa sobre un bosque mágico que había perdido sus sonidos por la contaminación"</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Producto+proceso narrados, sin mención de aprendizaje del estudiante</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ejemplo_centrado_producto_proceso</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Secuencia de "seres vivos" armada con NotebookLM para una colega, a partir del diseño curricular [08:20]-[09:30]</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Producto+proceso, sin aprendizaje articulado</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ejemplo_centrado_producto_proceso</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Evaluación adaptada para alumna con dificultades, IA generó versión de desarrollo [14:59]-[15:46]</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Proceso de adaptación, sin resultado de aprendizaje articulado</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ejemplo_centrado_producto_proceso</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Proyecto colaborativo 4 grados: IA estructuró actos de obra sobre Roald Dahl para coordinar escritura grupal [22:28]-[23:43]</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Producto+proceso, sin aprendizaje articulado</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ejemplo_centrado_producto_proceso</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Actividad reparatoria armada con ChatGPT para alumno que no sabe leer/escribir [18:52]-[19:31]</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Proceso de adaptación, sin resultado de aprendizaje articulado</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>ejemplo_centrado_producto_proceso</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Teatro de sombras: figuras + archivo 3D con Gemini + impresión [04:26]-[06:12]</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Producto+proceso, sin aprendizaje articulado</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>ejemplo_centrado_producto_proceso</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>"Doble estructura" para cuentos: alumno crea, IA crea, se comparan [09:01]-[09:30]</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>El más cercano a articular aprendizaje -- describe intención del diseño, no resultado observado</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>estrategia_deteccion_uso_estudiantil</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Colega insertó palabra oculta en texto blanco; alumnos que copiaron de IA repitieron la palabra sin darse cuenta [21:58]-[25:09]</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>HALLAZGO: evidencia observada de que el aprendizaje NO ocurrió -- no encaja en ninguno de los dos códigos nuevos, se nombra aparte (ver relectura_producto_proceso_aprendizaje.md §3)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Add criterio_etario_ciclo / criterio_heterogeneidad_grupo, correct prior claim
Splits criterio_contextual_grupo into three distinct phenomena per the
researcher's request. Full-corpus reread finds a real tension, not the
uniform exclusion pattern I claimed in the previous turn based only on
P1 and P15: 4 participants lean exclusionary (P1, P6, P9, P15), 3
explicitly reject that logic (P3, P4 -- "independientemente del
grado" --, P12 -- adapts via unplugged-first work in first grade
instead of excluding it). criterio_heterogeneidad_competencias_grupo
stays thin (1/15, P14 only) -- not forced. P7/P8 reclassified as
individual-student adaptation, already covered by
adaptacion_saberes_previos, removed from this count.
</commit_message>
<xml_diff>
--- a/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
+++ b/quality_reports/strategy/ia-generativa-docentes-primaria/codebook_v0_ia-generativa-docentes-primaria.xlsx
@@ -3157,7 +3157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3287,6 +3287,40 @@
       <c r="D8" s="28" t="inlineStr">
         <is>
           <t>"Me gusta que mis planificaciones sean mías". Código de alta carga identitaria -- anotar si la tensión se resuelve a favor de la IA, de la docente, o queda sin resolver. Puede coexistir con competencia_critica_reflexiva (Núcleo 3). Ref.: Moscovici (1986); Castañeda, Postigo-Fuentes &amp; Arroyo-Sagasta (2025, REEC 48 extra) -- verificada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>criterio_etario_ciclo (inductivo, 2026-08-07)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>La docente toma decisiones sobre el uso de IAG en función del ciclo/edad (primer ciclo 1-3 vs. segundo ciclo 4-7); incluye exclusión y contra-instancias explícitas.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Menciona el ciclo/edad como razón para usar, no usar, o adaptar el uso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>criterio_heterogeneidad_competencias_grupo (inductivo, 2026-08-07)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>La docente considera la heterogeneidad de competencias digitales dentro de un mismo grupo/grado (no por ciclo).</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Diferencias de manejo técnico entre compañeros del mismo grado como variable de planificación.</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4127,6 +4161,60 @@
       <c r="E33" t="inlineStr">
         <is>
           <t>Búsqueda activa en relectura corpus completo: 0/15 -- ausencia real, buscada, no solo constatada por omisión</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>criterio_etario_ciclo</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Ciclo/edad como criterio explícito de uso, no uso, o adaptación de IAG -- incluye exclusión y contra-instancias.</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Núcleo 5</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Relectura corpus completo: 7/15, dividido 4 exclusión (P1,P6,P9,P15) / 3 contra-instancia (P3,P4,P12) -- corrige lectura previa que asumía consenso solo con P1/P15</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>criterio_heterogeneidad_competencias_grupo</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Heterogeneidad de competencias digitales dentro de un mismo grupo/grado, distinto de ciclo.</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Núcleo 5</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Relectura corpus completo: 1/15 (P14) -- código delgado, no forzado</t>
         </is>
       </c>
     </row>
@@ -4145,7 +4233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E111"/>
+  <dimension ref="A1:E117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6949,6 +7037,168 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>criterio_etario_ciclo</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>"Confirma que lo aplicaría también en primer ciclo (1° y 2°/3° grado)"</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>CONTRA-INSTANCIA -- rechaza el ciclo como criterio de exclusión</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>criterio_etario_ciclo</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>"La incluiría también en primer ciclo... se puede sumar tranquilamente a cualquier tipo de planificación... independientemente del grado" [línea 72]</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>CONTRA-INSTANCIA explícita, la más nítida del corpus</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>criterio_etario_ciclo</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>"Con grados chicos en contextos vulnerables cuesta más, es todo más de cero"</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Exclusión mixta -- edad + vulnerabilidad socioeconómica, no criterio etario puro</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>criterio_etario_ciclo</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>"Cree que es más apropiada para segundo ciclo que primer ciclo" [20:26]</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Exclusión relativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>criterio_etario_ciclo</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Primer grado: trabajo "desenchufado" primero, luego animación vía IA; grados mayores: curaduría directa [11:17-12:40]</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>ADAPTACIÓN DIFERENCIADA -- no excluye, adapta el tipo de actividad por ciclo</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>criterio_heterogeneidad_competencias_grupo</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>"Hay alumnos que pueden arrastrar muy bien bloques... y otros que no, entonces lograr que todos vayan a la par lleva tiempo"</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Única instancia clara del corpus -- código delgado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>